<commit_message>
Refreshed latest betting odds
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -224,6 +224,48 @@
   </si>
   <si>
     <t>500:1</t>
+  </si>
+  <si>
+    <t>5:2</t>
+  </si>
+  <si>
+    <t>9:2</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>5:1</t>
+  </si>
+  <si>
+    <t>15:2</t>
+  </si>
+  <si>
+    <t>17:2</t>
+  </si>
+  <si>
+    <t>9:1</t>
+  </si>
+  <si>
+    <t>14:1</t>
+  </si>
+  <si>
+    <t>125:1</t>
+  </si>
+  <si>
+    <t>150:1</t>
+  </si>
+  <si>
+    <t>1000:1</t>
+  </si>
+  <si>
+    <t>500:11500</t>
+  </si>
+  <si>
+    <t>1500:</t>
+  </si>
+  <si>
+    <t>1500:1</t>
   </si>
 </sst>
 </file>
@@ -254,12 +296,20 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
     </fill>
   </fills>
   <borders count="1">
@@ -281,7 +331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -305,6 +355,8 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -674,8 +726,9 @@
         <v>1</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>59</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="F2" s="10"/>
       <c r="G2" s="10"/>
     </row>
     <row r="3">
@@ -692,8 +745,9 @@
         <v>1</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>60</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="F3" s="10"/>
       <c r="G3" s="10"/>
     </row>
     <row r="4">
@@ -710,8 +764,9 @@
         <v>1</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>57</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="F4" s="10"/>
       <c r="G4" s="10"/>
     </row>
     <row r="5">
@@ -728,8 +783,9 @@
         <v>1</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>60</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="F5" s="10"/>
       <c r="G5" s="10"/>
     </row>
     <row r="6">
@@ -746,8 +802,9 @@
         <v>1</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>58</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
     <row r="7">
@@ -764,8 +821,9 @@
         <v>1</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>64</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="F7" s="10"/>
       <c r="G7" s="10"/>
     </row>
     <row r="8">
@@ -782,8 +840,9 @@
         <v>1</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>63</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="F8" s="10"/>
       <c r="G8" s="10"/>
     </row>
     <row r="9">
@@ -800,8 +859,9 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>62</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="F9" s="10"/>
       <c r="G9" s="10"/>
     </row>
     <row r="10">
@@ -818,8 +878,9 @@
         <v>1</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>66</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="F10" s="10"/>
       <c r="G10" s="10"/>
     </row>
     <row r="11">
@@ -836,8 +897,9 @@
         <v>1</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>66</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="F11" s="10"/>
       <c r="G11" s="10"/>
     </row>
     <row r="12">
@@ -854,8 +916,9 @@
         <v>1</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>67</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="F12" s="10"/>
       <c r="G12" s="10"/>
     </row>
     <row r="13">
@@ -872,8 +935,9 @@
         <v>1</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>69</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F13" s="10"/>
       <c r="G13" s="10"/>
     </row>
     <row r="14">
@@ -890,8 +954,9 @@
         <v>1</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>61</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="F14" s="10"/>
       <c r="G14" s="10"/>
     </row>
     <row r="15">
@@ -908,8 +973,9 @@
         <v>1</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>66</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F15" s="10"/>
       <c r="G15" s="10"/>
     </row>
     <row r="16">
@@ -926,8 +992,9 @@
         <v>1</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>68</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F16" s="10"/>
       <c r="G16" s="10"/>
     </row>
     <row r="17">
@@ -944,8 +1011,9 @@
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>68</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F17" s="10"/>
       <c r="G17" s="10"/>
     </row>
     <row r="18">
@@ -964,6 +1032,7 @@
       <c r="E18" s="10" t="s">
         <v>70</v>
       </c>
+      <c r="F18" s="10"/>
       <c r="G18" s="10"/>
     </row>
     <row r="19">
@@ -980,8 +1049,9 @@
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>70</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="F19" s="10"/>
       <c r="G19" s="10"/>
     </row>
     <row r="20">
@@ -998,8 +1068,9 @@
         <v>1</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>65</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="F20" s="10"/>
       <c r="G20" s="10"/>
     </row>
     <row r="21">
@@ -1016,8 +1087,9 @@
         <v>1</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>69</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F21" s="10"/>
       <c r="G21" s="10"/>
     </row>
     <row r="22">
@@ -1036,6 +1108,7 @@
       <c r="E22" s="10" t="s">
         <v>70</v>
       </c>
+      <c r="F22" s="10"/>
       <c r="G22" s="10"/>
     </row>
     <row r="23">
@@ -1052,8 +1125,9 @@
         <v>1</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>70</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="F23" s="10"/>
       <c r="G23" s="10"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update prices and team names for 2026 season
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -266,6 +266,12 @@
   </si>
   <si>
     <t>1500:1</t>
+  </si>
+  <si>
+    <t>7:1</t>
+  </si>
+  <si>
+    <t>AUD</t>
   </si>
 </sst>
 </file>
@@ -840,7 +846,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
@@ -916,7 +922,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
@@ -954,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -992,7 +998,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
@@ -1011,7 +1017,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
@@ -1020,8 +1026,8 @@
       <c r="A18" t="s">
         <v>29</v>
       </c>
-      <c r="B18" t="s">
-        <v>30</v>
+      <c r="B18" s="0" t="s">
+        <v>86</v>
       </c>
       <c r="C18">
         <v>2026</v>
@@ -1039,8 +1045,8 @@
       <c r="A19" t="s">
         <v>31</v>
       </c>
-      <c r="B19" t="s">
-        <v>30</v>
+      <c r="B19" s="0" t="s">
+        <v>86</v>
       </c>
       <c r="C19">
         <v>2026</v>
@@ -1049,7 +1055,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
@@ -1106,7 +1112,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>

</xml_diff>

<commit_message>
Updated betting odds pre-race 1, FastF1 API updates
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -272,6 +272,24 @@
   </si>
   <si>
     <t>AUD</t>
+  </si>
+  <si>
+    <t>Odds_Pre_Weekend</t>
+  </si>
+  <si>
+    <t>Odds_Pre_Quali</t>
+  </si>
+  <si>
+    <t>Odds_Post_FP2</t>
+  </si>
+  <si>
+    <t>1000/1</t>
+  </si>
+  <si>
+    <t>3000/1</t>
+  </si>
+  <si>
+    <t>750/1</t>
   </si>
 </sst>
 </file>
@@ -691,8 +709,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <cols>
     <col min="5" max="5" style="5"/>
-    <col min="6" max="6" width="15.74" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14.12" style="10" customWidth="1"/>
+    <col min="6" max="6" width="22.06" style="10" customWidth="1"/>
+    <col min="7" max="7" width="17.65" style="10" customWidth="1"/>
+    <col min="8" max="8" width="17.94" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -712,10 +731,13 @@
         <v>4</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>38</v>
+        <v>87</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>39</v>
+        <v>88</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="2">
@@ -731,11 +753,16 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="2">
+        <v>46036</v>
+      </c>
+      <c r="F2" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="10"/>
       <c r="G2" s="10"/>
+      <c r="H2" s="2">
+        <v>46036</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -750,11 +777,16 @@
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="2">
+        <v>46032</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="F3" s="10"/>
       <c r="G3" s="10"/>
+      <c r="H3" s="2">
+        <v>46032</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -769,11 +801,16 @@
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="2">
+        <v>46121</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="F4" s="10"/>
       <c r="G4" s="10"/>
+      <c r="H4" s="2">
+        <v>46121</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
@@ -788,11 +825,16 @@
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="2">
+        <v>46068</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="10"/>
       <c r="G5" s="10"/>
+      <c r="H5" s="2">
+        <v>46068</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -807,11 +849,16 @@
       <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="2">
+        <v>46028</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="10"/>
       <c r="G6" s="10"/>
+      <c r="H6" s="2">
+        <v>46028</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
@@ -826,11 +873,16 @@
       <c r="D7">
         <v>1</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F7" s="10"/>
       <c r="G7" s="10"/>
+      <c r="H7" s="5" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
@@ -845,11 +897,16 @@
       <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="2">
+        <v>46032</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F8" s="10"/>
       <c r="G8" s="10"/>
+      <c r="H8" s="2">
+        <v>46032</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
@@ -864,11 +921,16 @@
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="2">
+        <v>46027</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="10"/>
       <c r="G9" s="10"/>
+      <c r="H9" s="2">
+        <v>46027</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
@@ -883,11 +945,16 @@
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="10"/>
       <c r="G10" s="10"/>
+      <c r="H10" s="5" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
@@ -902,11 +969,16 @@
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="10"/>
       <c r="G11" s="10"/>
+      <c r="H11" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
@@ -921,11 +993,16 @@
       <c r="D12">
         <v>1</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F12" s="10"/>
       <c r="G12" s="10"/>
+      <c r="H12" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
@@ -940,11 +1017,16 @@
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="10"/>
       <c r="G13" s="10"/>
+      <c r="H13" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
@@ -959,11 +1041,16 @@
       <c r="D14">
         <v>1</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F14" s="10"/>
       <c r="G14" s="10"/>
+      <c r="H14" s="5" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
@@ -978,11 +1065,16 @@
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F15" s="10"/>
       <c r="G15" s="10"/>
+      <c r="H15" s="5" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
@@ -997,11 +1089,16 @@
       <c r="D16">
         <v>1</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="5">
+        <v>5001</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F16" s="10"/>
       <c r="G16" s="10"/>
+      <c r="H16" s="5">
+        <v>5001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
@@ -1016,11 +1113,16 @@
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="10"/>
       <c r="G17" s="10"/>
+      <c r="H17" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
@@ -1035,11 +1137,16 @@
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F18" s="10"/>
       <c r="G18" s="10"/>
+      <c r="H18" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
@@ -1054,11 +1161,16 @@
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F19" s="10"/>
       <c r="G19" s="10"/>
+      <c r="H19" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
@@ -1073,11 +1185,16 @@
       <c r="D20">
         <v>1</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="10"/>
       <c r="G20" s="10"/>
+      <c r="H20" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
@@ -1092,11 +1209,16 @@
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="F21" s="10"/>
       <c r="G21" s="10"/>
+      <c r="H21" s="5" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
@@ -1111,11 +1233,16 @@
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="F22" s="10"/>
       <c r="G22" s="10"/>
+      <c r="H22" s="5" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
@@ -1130,11 +1257,16 @@
       <c r="D23">
         <v>1</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F23" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="F23" s="10"/>
       <c r="G23" s="10"/>
+      <c r="H23" s="5" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
Final odds for 2026 race 1
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -291,12 +291,54 @@
   <si>
     <t>750/1</t>
   </si>
+  <si>
+    <t>14-1</t>
+  </si>
+  <si>
+    <t>10-1</t>
+  </si>
+  <si>
+    <t>9-4</t>
+  </si>
+  <si>
+    <t>15-2</t>
+  </si>
+  <si>
+    <t>6-1</t>
+  </si>
+  <si>
+    <t>80-1</t>
+  </si>
+  <si>
+    <t>5-1</t>
+  </si>
+  <si>
+    <t>750-1</t>
+  </si>
+  <si>
+    <t>500-1</t>
+  </si>
+  <si>
+    <t>400-1</t>
+  </si>
+  <si>
+    <t>3000-1</t>
+  </si>
+  <si>
+    <t>1000-1</t>
+  </si>
+  <si>
+    <t>"14-1"</t>
+  </si>
+  <si>
+    <t>"14-1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="8" mc:Ignorable="x14ac">
-  <numFmts count="9">
+  <numFmts count="11">
     <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);(&quot;$&quot;#,##0)"/>
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red](&quot;$&quot;#,##0)"/>
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);(&quot;$&quot;#,##0.00)"/>
@@ -306,6 +348,8 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* (#,##0.00);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* (#,##0.00);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="d/m"/>
+    <numFmt numFmtId="165" formatCode="0E+00"/>
+    <numFmt numFmtId="166" formatCode="hh:mm"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -355,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -381,6 +425,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -753,8 +802,8 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="2">
-        <v>46036</v>
+      <c r="E2" s="10" t="s">
+        <v>93</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>77</v>
@@ -763,6 +812,7 @@
       <c r="H2" s="2">
         <v>46036</v>
       </c>
+      <c r="J2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -777,8 +827,8 @@
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3" s="2">
-        <v>46032</v>
+      <c r="E3" s="10" t="s">
+        <v>94</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>78</v>
@@ -801,8 +851,8 @@
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="2">
-        <v>46121</v>
+      <c r="E4" s="10" t="s">
+        <v>95</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>71</v>
@@ -825,8 +875,8 @@
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" s="2">
-        <v>46068</v>
+      <c r="E5" s="10" t="s">
+        <v>96</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>76</v>
@@ -849,8 +899,8 @@
       <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6" s="2">
-        <v>46028</v>
+      <c r="E6" s="10" t="s">
+        <v>97</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>72</v>
@@ -873,8 +923,8 @@
       <c r="D7">
         <v>1</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>42</v>
+      <c r="E7" s="10" t="s">
+        <v>98</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>66</v>
@@ -897,8 +947,8 @@
       <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" s="2">
-        <v>46032</v>
+      <c r="E8" s="10" t="s">
+        <v>94</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>85</v>
@@ -921,8 +971,8 @@
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9" s="2">
-        <v>46027</v>
+      <c r="E9" s="10" t="s">
+        <v>99</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>74</v>
@@ -945,8 +995,8 @@
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>92</v>
+      <c r="E10" s="10" t="s">
+        <v>100</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>69</v>
@@ -969,8 +1019,8 @@
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>46</v>
+      <c r="E11" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>69</v>
@@ -993,8 +1043,8 @@
       <c r="D12">
         <v>1</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>46</v>
+      <c r="E12" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>70</v>
@@ -1017,8 +1067,8 @@
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>44</v>
+      <c r="E13" s="10" t="s">
+        <v>102</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>70</v>
@@ -1041,8 +1091,8 @@
       <c r="D14">
         <v>1</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>91</v>
+      <c r="E14" s="10" t="s">
+        <v>103</v>
       </c>
       <c r="F14" s="10" t="s">
         <v>69</v>
@@ -1065,8 +1115,8 @@
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>91</v>
+      <c r="E15" s="10" t="s">
+        <v>103</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>70</v>
@@ -1089,15 +1139,15 @@
       <c r="D16">
         <v>1</v>
       </c>
-      <c r="E16" s="5">
-        <v>5001</v>
+      <c r="E16" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F16" s="10" t="s">
         <v>69</v>
       </c>
       <c r="G16" s="10"/>
-      <c r="H16" s="5">
-        <v>5001</v>
+      <c r="H16" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="17">
@@ -1113,8 +1163,8 @@
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>46</v>
+      <c r="E17" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>69</v>
@@ -1137,8 +1187,8 @@
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>46</v>
+      <c r="E18" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>70</v>
@@ -1161,8 +1211,8 @@
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>46</v>
+      <c r="E19" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>70</v>
@@ -1185,8 +1235,8 @@
       <c r="D20">
         <v>1</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>46</v>
+      <c r="E20" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>79</v>
@@ -1209,8 +1259,8 @@
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>90</v>
+      <c r="E21" s="10" t="s">
+        <v>104</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>70</v>
@@ -1233,8 +1283,8 @@
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>91</v>
+      <c r="E22" s="10" t="s">
+        <v>103</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>84</v>
@@ -1257,8 +1307,8 @@
       <c r="D23">
         <v>1</v>
       </c>
-      <c r="E23" s="5" t="s">
-        <v>91</v>
+      <c r="E23" s="10" t="s">
+        <v>103</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>81</v>

</xml_diff>

<commit_message>
Updated data and teams for Aus and China GPs, added copilot instructions
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -332,6 +332,24 @@
   </si>
   <si>
     <t>"14-1</t>
+  </si>
+  <si>
+    <t>6-4</t>
+  </si>
+  <si>
+    <t>11-4</t>
+  </si>
+  <si>
+    <t>66-1</t>
+  </si>
+  <si>
+    <t>100-1</t>
+  </si>
+  <si>
+    <t>1500-1</t>
+  </si>
+  <si>
+    <t>2000-1</t>
   </si>
 </sst>
 </file>
@@ -1318,6 +1336,446 @@
         <v>91</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24">
+        <v>2026</v>
+      </c>
+      <c r="D24" s="0">
+        <v>2</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25">
+        <v>2026</v>
+      </c>
+      <c r="D25" s="0">
+        <v>2</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26">
+        <v>2026</v>
+      </c>
+      <c r="D26" s="0">
+        <v>2</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27">
+        <v>2026</v>
+      </c>
+      <c r="D27" s="0">
+        <v>2</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28">
+        <v>2026</v>
+      </c>
+      <c r="D28" s="0">
+        <v>2</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="0">
+        <v>2</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30">
+        <v>2026</v>
+      </c>
+      <c r="D30" s="0">
+        <v>2</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31">
+        <v>2026</v>
+      </c>
+      <c r="D31" s="0">
+        <v>2</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32">
+        <v>2026</v>
+      </c>
+      <c r="D32" s="0">
+        <v>2</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33">
+        <v>2026</v>
+      </c>
+      <c r="D33" s="0">
+        <v>2</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34">
+        <v>2026</v>
+      </c>
+      <c r="D34" s="0">
+        <v>2</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35">
+        <v>2026</v>
+      </c>
+      <c r="D35" s="0">
+        <v>2</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36">
+        <v>2026</v>
+      </c>
+      <c r="D36" s="0">
+        <v>2</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37">
+        <v>2026</v>
+      </c>
+      <c r="D37" s="0">
+        <v>2</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38">
+        <v>2026</v>
+      </c>
+      <c r="D38" s="0">
+        <v>2</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>28</v>
+      </c>
+      <c r="B39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39">
+        <v>2026</v>
+      </c>
+      <c r="D39" s="0">
+        <v>2</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>29</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40">
+        <v>2026</v>
+      </c>
+      <c r="D40" s="0">
+        <v>2</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41">
+        <v>2026</v>
+      </c>
+      <c r="D41" s="0">
+        <v>2</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>32</v>
+      </c>
+      <c r="B42" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42">
+        <v>2026</v>
+      </c>
+      <c r="D42" s="0">
+        <v>2</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43">
+        <v>2026</v>
+      </c>
+      <c r="D43" s="0">
+        <v>2</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>35</v>
+      </c>
+      <c r="B44" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44">
+        <v>2026</v>
+      </c>
+      <c r="D44" s="0">
+        <v>2</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45">
+        <v>2026</v>
+      </c>
+      <c r="D45" s="0">
+        <v>2</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated betting odds post race 3
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -350,6 +350,30 @@
   </si>
   <si>
     <t>2000-1</t>
+  </si>
+  <si>
+    <t>10-11</t>
+  </si>
+  <si>
+    <t>9-5</t>
+  </si>
+  <si>
+    <t>16-1</t>
+  </si>
+  <si>
+    <t>20-1</t>
+  </si>
+  <si>
+    <t>33-1</t>
+  </si>
+  <si>
+    <t>50-1</t>
+  </si>
+  <si>
+    <t>250-1</t>
+  </si>
+  <si>
+    <t>2500-1</t>
   </si>
 </sst>
 </file>
@@ -1776,6 +1800,446 @@
         <v>103</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46">
+        <v>2026</v>
+      </c>
+      <c r="D46" s="0">
+        <v>3</v>
+      </c>
+      <c r="E46" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="H46" s="0" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47">
+        <v>2026</v>
+      </c>
+      <c r="D47" s="0">
+        <v>3</v>
+      </c>
+      <c r="E47" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="H47" s="0" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>8</v>
+      </c>
+      <c r="B48" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48">
+        <v>2026</v>
+      </c>
+      <c r="D48" s="0">
+        <v>3</v>
+      </c>
+      <c r="E48" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="H48" s="0" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>10</v>
+      </c>
+      <c r="B49" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49">
+        <v>2026</v>
+      </c>
+      <c r="D49" s="0">
+        <v>3</v>
+      </c>
+      <c r="E49" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="H49" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50">
+        <v>2026</v>
+      </c>
+      <c r="D50" s="0">
+        <v>3</v>
+      </c>
+      <c r="E50" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="H50" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51">
+        <v>2026</v>
+      </c>
+      <c r="D51" s="0">
+        <v>3</v>
+      </c>
+      <c r="E51" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H51" s="0" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>14</v>
+      </c>
+      <c r="B52" t="s">
+        <v>15</v>
+      </c>
+      <c r="C52">
+        <v>2026</v>
+      </c>
+      <c r="D52" s="0">
+        <v>3</v>
+      </c>
+      <c r="E52" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="H52" s="0" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>16</v>
+      </c>
+      <c r="B53" t="s">
+        <v>15</v>
+      </c>
+      <c r="C53">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="0">
+        <v>3</v>
+      </c>
+      <c r="E53" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="H53" s="0" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>17</v>
+      </c>
+      <c r="B54" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54">
+        <v>2026</v>
+      </c>
+      <c r="D54" s="0">
+        <v>3</v>
+      </c>
+      <c r="E54" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H54" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55">
+        <v>2026</v>
+      </c>
+      <c r="D55" s="0">
+        <v>3</v>
+      </c>
+      <c r="E55" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H55" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56">
+        <v>2026</v>
+      </c>
+      <c r="D56" s="0">
+        <v>3</v>
+      </c>
+      <c r="E56" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="H56" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>22</v>
+      </c>
+      <c r="B57" t="s">
+        <v>21</v>
+      </c>
+      <c r="C57">
+        <v>2026</v>
+      </c>
+      <c r="D57" s="0">
+        <v>3</v>
+      </c>
+      <c r="E57" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="H57" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>23</v>
+      </c>
+      <c r="B58" t="s">
+        <v>24</v>
+      </c>
+      <c r="C58">
+        <v>2026</v>
+      </c>
+      <c r="D58" s="0">
+        <v>3</v>
+      </c>
+      <c r="E58" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H58" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>25</v>
+      </c>
+      <c r="B59" t="s">
+        <v>24</v>
+      </c>
+      <c r="C59">
+        <v>2026</v>
+      </c>
+      <c r="D59" s="0">
+        <v>3</v>
+      </c>
+      <c r="E59" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H59" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>26</v>
+      </c>
+      <c r="B60" t="s">
+        <v>27</v>
+      </c>
+      <c r="C60">
+        <v>2026</v>
+      </c>
+      <c r="D60" s="0">
+        <v>3</v>
+      </c>
+      <c r="E60" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="H60" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61">
+        <v>2026</v>
+      </c>
+      <c r="D61" s="0">
+        <v>3</v>
+      </c>
+      <c r="E61" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="H61" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>29</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C62">
+        <v>2026</v>
+      </c>
+      <c r="D62" s="0">
+        <v>3</v>
+      </c>
+      <c r="E62" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H62" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>31</v>
+      </c>
+      <c r="B63" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C63">
+        <v>2026</v>
+      </c>
+      <c r="D63" s="0">
+        <v>3</v>
+      </c>
+      <c r="E63" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H63" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>32</v>
+      </c>
+      <c r="B64" t="s">
+        <v>33</v>
+      </c>
+      <c r="C64">
+        <v>2026</v>
+      </c>
+      <c r="D64" s="0">
+        <v>3</v>
+      </c>
+      <c r="E64" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="H64" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>34</v>
+      </c>
+      <c r="B65" t="s">
+        <v>33</v>
+      </c>
+      <c r="C65">
+        <v>2026</v>
+      </c>
+      <c r="D65" s="0">
+        <v>3</v>
+      </c>
+      <c r="E65" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H65" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>35</v>
+      </c>
+      <c r="B66" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66">
+        <v>2026</v>
+      </c>
+      <c r="D66" s="0">
+        <v>3</v>
+      </c>
+      <c r="E66" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H66" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>37</v>
+      </c>
+      <c r="B67" t="s">
+        <v>36</v>
+      </c>
+      <c r="C67">
+        <v>2026</v>
+      </c>
+      <c r="D67" s="0">
+        <v>3</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="H67" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated pre-race betting odds for Canada
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -374,6 +374,36 @@
   </si>
   <si>
     <t>2500-1</t>
+  </si>
+  <si>
+    <t>Odds_Post_Quali</t>
+  </si>
+  <si>
+    <t>4000-1</t>
+  </si>
+  <si>
+    <t>29-10</t>
+  </si>
+  <si>
+    <t>9-1</t>
+  </si>
+  <si>
+    <t>11-1</t>
+  </si>
+  <si>
+    <t>25-1</t>
+  </si>
+  <si>
+    <t>2-1</t>
+  </si>
+  <si>
+    <t>23-10</t>
+  </si>
+  <si>
+    <t>18-1</t>
+  </si>
+  <si>
+    <t>28-1</t>
   </si>
 </sst>
 </file>
@@ -803,6 +833,7 @@
     <col min="6" max="6" width="22.06" style="10" customWidth="1"/>
     <col min="7" max="7" width="17.65" style="10" customWidth="1"/>
     <col min="8" max="8" width="17.94" customWidth="1"/>
+    <col min="9" max="9" width="18.43" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -830,6 +861,9 @@
       <c r="H1" s="9" t="s">
         <v>89</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -2240,6 +2274,820 @@
         <v>120</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>5</v>
+      </c>
+      <c r="B68" t="s">
+        <v>6</v>
+      </c>
+      <c r="C68">
+        <v>2026</v>
+      </c>
+      <c r="D68" s="0">
+        <v>4</v>
+      </c>
+      <c r="E68" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="I68" s="0" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B69" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69">
+        <v>2026</v>
+      </c>
+      <c r="D69" s="0">
+        <v>4</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>8</v>
+      </c>
+      <c r="B70" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70">
+        <v>2026</v>
+      </c>
+      <c r="D70" s="0">
+        <v>4</v>
+      </c>
+      <c r="E70" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="I70" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>10</v>
+      </c>
+      <c r="B71" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71">
+        <v>2026</v>
+      </c>
+      <c r="D71" s="0">
+        <v>4</v>
+      </c>
+      <c r="E71" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="I71" s="0" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>11</v>
+      </c>
+      <c r="B72" t="s">
+        <v>12</v>
+      </c>
+      <c r="C72">
+        <v>2026</v>
+      </c>
+      <c r="D72" s="0">
+        <v>4</v>
+      </c>
+      <c r="E72" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="I72" s="0" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>13</v>
+      </c>
+      <c r="B73" t="s">
+        <v>12</v>
+      </c>
+      <c r="C73">
+        <v>2026</v>
+      </c>
+      <c r="D73" s="0">
+        <v>4</v>
+      </c>
+      <c r="E73" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="I73" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>14</v>
+      </c>
+      <c r="B74" t="s">
+        <v>15</v>
+      </c>
+      <c r="C74">
+        <v>2026</v>
+      </c>
+      <c r="D74" s="0">
+        <v>4</v>
+      </c>
+      <c r="E74" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="I74" s="0" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>16</v>
+      </c>
+      <c r="B75" t="s">
+        <v>15</v>
+      </c>
+      <c r="C75">
+        <v>2026</v>
+      </c>
+      <c r="D75" s="0">
+        <v>4</v>
+      </c>
+      <c r="E75" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="I75" s="0" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>17</v>
+      </c>
+      <c r="B76" t="s">
+        <v>18</v>
+      </c>
+      <c r="C76">
+        <v>2026</v>
+      </c>
+      <c r="D76" s="0">
+        <v>4</v>
+      </c>
+      <c r="E76" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="I76" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>19</v>
+      </c>
+      <c r="B77" t="s">
+        <v>18</v>
+      </c>
+      <c r="C77">
+        <v>2026</v>
+      </c>
+      <c r="D77" s="0">
+        <v>4</v>
+      </c>
+      <c r="E77" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="I77" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>20</v>
+      </c>
+      <c r="B78" t="s">
+        <v>21</v>
+      </c>
+      <c r="C78">
+        <v>2026</v>
+      </c>
+      <c r="D78" s="0">
+        <v>4</v>
+      </c>
+      <c r="E78" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="I78" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>22</v>
+      </c>
+      <c r="B79" t="s">
+        <v>21</v>
+      </c>
+      <c r="C79">
+        <v>2026</v>
+      </c>
+      <c r="D79" s="0">
+        <v>4</v>
+      </c>
+      <c r="E79" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="I79" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>23</v>
+      </c>
+      <c r="B80" t="s">
+        <v>24</v>
+      </c>
+      <c r="C80">
+        <v>2026</v>
+      </c>
+      <c r="D80" s="0">
+        <v>4</v>
+      </c>
+      <c r="E80" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="I80" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>25</v>
+      </c>
+      <c r="B81" t="s">
+        <v>24</v>
+      </c>
+      <c r="C81">
+        <v>2026</v>
+      </c>
+      <c r="D81" s="0">
+        <v>4</v>
+      </c>
+      <c r="E81" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="I81" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>26</v>
+      </c>
+      <c r="B82" t="s">
+        <v>27</v>
+      </c>
+      <c r="C82">
+        <v>2026</v>
+      </c>
+      <c r="D82" s="0">
+        <v>4</v>
+      </c>
+      <c r="E82" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="I82" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>28</v>
+      </c>
+      <c r="B83" t="s">
+        <v>27</v>
+      </c>
+      <c r="C83">
+        <v>2026</v>
+      </c>
+      <c r="D83" s="0">
+        <v>4</v>
+      </c>
+      <c r="E83" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="I83" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>29</v>
+      </c>
+      <c r="B84" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C84">
+        <v>2026</v>
+      </c>
+      <c r="D84" s="0">
+        <v>4</v>
+      </c>
+      <c r="E84" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="I84" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>31</v>
+      </c>
+      <c r="B85" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C85">
+        <v>2026</v>
+      </c>
+      <c r="D85" s="0">
+        <v>4</v>
+      </c>
+      <c r="E85" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="I85" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>32</v>
+      </c>
+      <c r="B86" t="s">
+        <v>33</v>
+      </c>
+      <c r="C86">
+        <v>2026</v>
+      </c>
+      <c r="D86" s="0">
+        <v>4</v>
+      </c>
+      <c r="E86" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I86" s="0" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s">
+        <v>34</v>
+      </c>
+      <c r="B87" t="s">
+        <v>33</v>
+      </c>
+      <c r="C87">
+        <v>2026</v>
+      </c>
+      <c r="D87" s="0">
+        <v>4</v>
+      </c>
+      <c r="E87" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I87" s="0" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s">
+        <v>35</v>
+      </c>
+      <c r="B88" t="s">
+        <v>36</v>
+      </c>
+      <c r="C88">
+        <v>2026</v>
+      </c>
+      <c r="D88" s="0">
+        <v>4</v>
+      </c>
+      <c r="E88" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="I88" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s">
+        <v>37</v>
+      </c>
+      <c r="B89" t="s">
+        <v>36</v>
+      </c>
+      <c r="C89">
+        <v>2026</v>
+      </c>
+      <c r="D89" s="0">
+        <v>4</v>
+      </c>
+      <c r="E89" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="I89" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s">
+        <v>5</v>
+      </c>
+      <c r="B90" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90">
+        <v>2026</v>
+      </c>
+      <c r="D90" s="0">
+        <v>5</v>
+      </c>
+      <c r="F90" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s">
+        <v>7</v>
+      </c>
+      <c r="B91" t="s">
+        <v>6</v>
+      </c>
+      <c r="C91">
+        <v>2026</v>
+      </c>
+      <c r="D91" s="0">
+        <v>5</v>
+      </c>
+      <c r="F91" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s">
+        <v>8</v>
+      </c>
+      <c r="B92" t="s">
+        <v>9</v>
+      </c>
+      <c r="C92">
+        <v>2026</v>
+      </c>
+      <c r="D92" s="0">
+        <v>5</v>
+      </c>
+      <c r="F92" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s">
+        <v>10</v>
+      </c>
+      <c r="B93" t="s">
+        <v>9</v>
+      </c>
+      <c r="C93">
+        <v>2026</v>
+      </c>
+      <c r="D93" s="0">
+        <v>5</v>
+      </c>
+      <c r="F93" s="10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s">
+        <v>11</v>
+      </c>
+      <c r="B94" t="s">
+        <v>12</v>
+      </c>
+      <c r="C94">
+        <v>2026</v>
+      </c>
+      <c r="D94" s="0">
+        <v>5</v>
+      </c>
+      <c r="F94" s="10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s">
+        <v>13</v>
+      </c>
+      <c r="B95" t="s">
+        <v>12</v>
+      </c>
+      <c r="C95">
+        <v>2026</v>
+      </c>
+      <c r="D95" s="0">
+        <v>5</v>
+      </c>
+      <c r="F95" s="10" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s">
+        <v>14</v>
+      </c>
+      <c r="B96" t="s">
+        <v>15</v>
+      </c>
+      <c r="C96">
+        <v>2026</v>
+      </c>
+      <c r="D96" s="0">
+        <v>5</v>
+      </c>
+      <c r="F96" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s">
+        <v>16</v>
+      </c>
+      <c r="B97" t="s">
+        <v>15</v>
+      </c>
+      <c r="C97">
+        <v>2026</v>
+      </c>
+      <c r="D97" s="0">
+        <v>5</v>
+      </c>
+      <c r="F97" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s">
+        <v>17</v>
+      </c>
+      <c r="B98" t="s">
+        <v>18</v>
+      </c>
+      <c r="C98">
+        <v>2026</v>
+      </c>
+      <c r="D98" s="0">
+        <v>5</v>
+      </c>
+      <c r="F98" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>19</v>
+      </c>
+      <c r="B99" t="s">
+        <v>18</v>
+      </c>
+      <c r="C99">
+        <v>2026</v>
+      </c>
+      <c r="D99" s="0">
+        <v>5</v>
+      </c>
+      <c r="F99" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s">
+        <v>20</v>
+      </c>
+      <c r="B100" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100">
+        <v>2026</v>
+      </c>
+      <c r="D100" s="0">
+        <v>5</v>
+      </c>
+      <c r="F100" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>22</v>
+      </c>
+      <c r="B101" t="s">
+        <v>21</v>
+      </c>
+      <c r="C101">
+        <v>2026</v>
+      </c>
+      <c r="D101" s="0">
+        <v>5</v>
+      </c>
+      <c r="F101" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s">
+        <v>23</v>
+      </c>
+      <c r="B102" t="s">
+        <v>24</v>
+      </c>
+      <c r="C102">
+        <v>2026</v>
+      </c>
+      <c r="D102" s="0">
+        <v>5</v>
+      </c>
+      <c r="F102" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s">
+        <v>25</v>
+      </c>
+      <c r="B103" t="s">
+        <v>24</v>
+      </c>
+      <c r="C103">
+        <v>2026</v>
+      </c>
+      <c r="D103" s="0">
+        <v>5</v>
+      </c>
+      <c r="F103" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s">
+        <v>26</v>
+      </c>
+      <c r="B104" t="s">
+        <v>27</v>
+      </c>
+      <c r="C104">
+        <v>2026</v>
+      </c>
+      <c r="D104" s="0">
+        <v>5</v>
+      </c>
+      <c r="F104" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>28</v>
+      </c>
+      <c r="B105" t="s">
+        <v>27</v>
+      </c>
+      <c r="C105">
+        <v>2026</v>
+      </c>
+      <c r="D105" s="0">
+        <v>5</v>
+      </c>
+      <c r="F105" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s">
+        <v>29</v>
+      </c>
+      <c r="B106" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C106">
+        <v>2026</v>
+      </c>
+      <c r="D106" s="0">
+        <v>5</v>
+      </c>
+      <c r="F106" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s">
+        <v>31</v>
+      </c>
+      <c r="B107" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C107">
+        <v>2026</v>
+      </c>
+      <c r="D107" s="0">
+        <v>5</v>
+      </c>
+      <c r="F107" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s">
+        <v>32</v>
+      </c>
+      <c r="B108" t="s">
+        <v>33</v>
+      </c>
+      <c r="C108">
+        <v>2026</v>
+      </c>
+      <c r="D108" s="0">
+        <v>5</v>
+      </c>
+      <c r="F108" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s">
+        <v>34</v>
+      </c>
+      <c r="B109" t="s">
+        <v>33</v>
+      </c>
+      <c r="C109">
+        <v>2026</v>
+      </c>
+      <c r="D109" s="0">
+        <v>5</v>
+      </c>
+      <c r="F109" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s">
+        <v>35</v>
+      </c>
+      <c r="B110" t="s">
+        <v>36</v>
+      </c>
+      <c r="C110">
+        <v>2026</v>
+      </c>
+      <c r="D110" s="0">
+        <v>5</v>
+      </c>
+      <c r="F110" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s">
+        <v>37</v>
+      </c>
+      <c r="B111" t="s">
+        <v>36</v>
+      </c>
+      <c r="C111">
+        <v>2026</v>
+      </c>
+      <c r="D111" s="0">
+        <v>5</v>
+      </c>
+      <c r="F111" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated race stats and betting odds after Monaco
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -404,6 +404,30 @@
   </si>
   <si>
     <t>28-1</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>200-1</t>
+  </si>
+  <si>
+    <t>12-</t>
+  </si>
+  <si>
+    <t>12-1</t>
+  </si>
+  <si>
+    <t>13-2</t>
+  </si>
+  <si>
+    <t>11-2</t>
+  </si>
+  <si>
+    <t>9-2</t>
   </si>
 </sst>
 </file>
@@ -2727,6 +2751,9 @@
       <c r="D90" s="0">
         <v>5</v>
       </c>
+      <c r="E90" s="10" t="s">
+        <v>99</v>
+      </c>
       <c r="F90" s="10" t="s">
         <v>99</v>
       </c>
@@ -2744,6 +2771,9 @@
       <c r="D91" s="0">
         <v>5</v>
       </c>
+      <c r="E91" s="10" t="s">
+        <v>125</v>
+      </c>
       <c r="F91" s="10" t="s">
         <v>125</v>
       </c>
@@ -2761,6 +2791,9 @@
       <c r="D92" s="0">
         <v>5</v>
       </c>
+      <c r="E92" s="10" t="s">
+        <v>128</v>
+      </c>
       <c r="F92" s="10" t="s">
         <v>128</v>
       </c>
@@ -2778,6 +2811,9 @@
       <c r="D93" s="0">
         <v>5</v>
       </c>
+      <c r="E93" s="10" t="s">
+        <v>127</v>
+      </c>
       <c r="F93" s="10" t="s">
         <v>127</v>
       </c>
@@ -2795,6 +2831,9 @@
       <c r="D94" s="0">
         <v>5</v>
       </c>
+      <c r="E94" s="10" t="s">
+        <v>124</v>
+      </c>
       <c r="F94" s="10" t="s">
         <v>124</v>
       </c>
@@ -2812,6 +2851,9 @@
       <c r="D95" s="0">
         <v>5</v>
       </c>
+      <c r="E95" s="10" t="s">
+        <v>102</v>
+      </c>
       <c r="F95" s="10" t="s">
         <v>102</v>
       </c>
@@ -2829,6 +2871,9 @@
       <c r="D96" s="0">
         <v>5</v>
       </c>
+      <c r="E96" s="10" t="s">
+        <v>130</v>
+      </c>
       <c r="F96" s="10" t="s">
         <v>130</v>
       </c>
@@ -2846,6 +2891,9 @@
       <c r="D97" s="0">
         <v>5</v>
       </c>
+      <c r="E97" s="10" t="s">
+        <v>129</v>
+      </c>
       <c r="F97" s="10" t="s">
         <v>129</v>
       </c>
@@ -2863,6 +2911,9 @@
       <c r="D98" s="0">
         <v>5</v>
       </c>
+      <c r="E98" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F98" s="10" t="s">
         <v>100</v>
       </c>
@@ -2880,6 +2931,9 @@
       <c r="D99" s="0">
         <v>5</v>
       </c>
+      <c r="E99" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F99" s="10" t="s">
         <v>100</v>
       </c>
@@ -2897,6 +2951,9 @@
       <c r="D100" s="0">
         <v>5</v>
       </c>
+      <c r="E100" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F100" s="10" t="s">
         <v>100</v>
       </c>
@@ -2914,6 +2971,9 @@
       <c r="D101" s="0">
         <v>5</v>
       </c>
+      <c r="E101" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F101" s="10" t="s">
         <v>100</v>
       </c>
@@ -2931,6 +2991,9 @@
       <c r="D102" s="0">
         <v>5</v>
       </c>
+      <c r="E102" s="10" t="s">
+        <v>104</v>
+      </c>
       <c r="F102" s="10" t="s">
         <v>104</v>
       </c>
@@ -2948,6 +3011,9 @@
       <c r="D103" s="0">
         <v>5</v>
       </c>
+      <c r="E103" s="10" t="s">
+        <v>112</v>
+      </c>
       <c r="F103" s="10" t="s">
         <v>112</v>
       </c>
@@ -2965,6 +3031,9 @@
       <c r="D104" s="0">
         <v>5</v>
       </c>
+      <c r="E104" s="10" t="s">
+        <v>101</v>
+      </c>
       <c r="F104" s="10" t="s">
         <v>101</v>
       </c>
@@ -2982,6 +3051,9 @@
       <c r="D105" s="0">
         <v>5</v>
       </c>
+      <c r="E105" s="10" t="s">
+        <v>101</v>
+      </c>
       <c r="F105" s="10" t="s">
         <v>101</v>
       </c>
@@ -2999,6 +3071,9 @@
       <c r="D106" s="0">
         <v>5</v>
       </c>
+      <c r="E106" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F106" s="10" t="s">
         <v>100</v>
       </c>
@@ -3016,6 +3091,9 @@
       <c r="D107" s="0">
         <v>5</v>
       </c>
+      <c r="E107" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F107" s="10" t="s">
         <v>100</v>
       </c>
@@ -3033,6 +3111,9 @@
       <c r="D108" s="0">
         <v>5</v>
       </c>
+      <c r="E108" s="10" t="s">
+        <v>101</v>
+      </c>
       <c r="F108" s="10" t="s">
         <v>101</v>
       </c>
@@ -3050,6 +3131,9 @@
       <c r="D109" s="0">
         <v>5</v>
       </c>
+      <c r="E109" s="10" t="s">
+        <v>101</v>
+      </c>
       <c r="F109" s="10" t="s">
         <v>101</v>
       </c>
@@ -3067,6 +3151,9 @@
       <c r="D110" s="0">
         <v>5</v>
       </c>
+      <c r="E110" s="10" t="s">
+        <v>112</v>
+      </c>
       <c r="F110" s="10" t="s">
         <v>112</v>
       </c>
@@ -3084,8 +3171,451 @@
       <c r="D111" s="0">
         <v>5</v>
       </c>
+      <c r="E111" s="10" t="s">
+        <v>112</v>
+      </c>
       <c r="F111" s="10" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s">
+        <v>5</v>
+      </c>
+      <c r="B112" t="s">
+        <v>6</v>
+      </c>
+      <c r="C112">
+        <v>2026</v>
+      </c>
+      <c r="D112" s="0">
+        <v>6</v>
+      </c>
+      <c r="E112" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="G112" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s">
+        <v>7</v>
+      </c>
+      <c r="B113" t="s">
+        <v>6</v>
+      </c>
+      <c r="C113">
+        <v>2026</v>
+      </c>
+      <c r="D113" s="0">
+        <v>6</v>
+      </c>
+      <c r="E113" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G113" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s">
+        <v>8</v>
+      </c>
+      <c r="B114" t="s">
+        <v>9</v>
+      </c>
+      <c r="C114">
+        <v>2026</v>
+      </c>
+      <c r="D114" s="0">
+        <v>6</v>
+      </c>
+      <c r="E114" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="G114" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s">
+        <v>10</v>
+      </c>
+      <c r="B115" t="s">
+        <v>9</v>
+      </c>
+      <c r="C115">
+        <v>2026</v>
+      </c>
+      <c r="D115" s="0">
+        <v>6</v>
+      </c>
+      <c r="E115" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="G115" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s">
+        <v>11</v>
+      </c>
+      <c r="B116" t="s">
+        <v>12</v>
+      </c>
+      <c r="C116">
+        <v>2026</v>
+      </c>
+      <c r="D116" s="0">
+        <v>6</v>
+      </c>
+      <c r="E116" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G116" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s">
+        <v>13</v>
+      </c>
+      <c r="B117" t="s">
+        <v>12</v>
+      </c>
+      <c r="C117">
+        <v>2026</v>
+      </c>
+      <c r="D117" s="0">
+        <v>6</v>
+      </c>
+      <c r="E117" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="G117" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>14</v>
+      </c>
+      <c r="B118" t="s">
+        <v>15</v>
+      </c>
+      <c r="C118">
+        <v>2026</v>
+      </c>
+      <c r="D118" s="0">
+        <v>6</v>
+      </c>
+      <c r="E118" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="G118" s="10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>16</v>
+      </c>
+      <c r="B119" t="s">
+        <v>15</v>
+      </c>
+      <c r="C119">
+        <v>2026</v>
+      </c>
+      <c r="D119" s="0">
+        <v>6</v>
+      </c>
+      <c r="E119" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="G119" s="10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>17</v>
+      </c>
+      <c r="B120" t="s">
+        <v>18</v>
+      </c>
+      <c r="C120">
+        <v>2026</v>
+      </c>
+      <c r="D120" s="0">
+        <v>6</v>
+      </c>
+      <c r="E120" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G120" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>19</v>
+      </c>
+      <c r="B121" t="s">
+        <v>18</v>
+      </c>
+      <c r="C121">
+        <v>2026</v>
+      </c>
+      <c r="D121" s="0">
+        <v>6</v>
+      </c>
+      <c r="E121" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G121" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>20</v>
+      </c>
+      <c r="B122" t="s">
+        <v>21</v>
+      </c>
+      <c r="C122">
+        <v>2026</v>
+      </c>
+      <c r="D122" s="0">
+        <v>6</v>
+      </c>
+      <c r="E122" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G122" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>22</v>
+      </c>
+      <c r="B123" t="s">
+        <v>21</v>
+      </c>
+      <c r="C123">
+        <v>2026</v>
+      </c>
+      <c r="D123" s="0">
+        <v>6</v>
+      </c>
+      <c r="E123" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G123" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>23</v>
+      </c>
+      <c r="B124" t="s">
+        <v>24</v>
+      </c>
+      <c r="C124">
+        <v>2026</v>
+      </c>
+      <c r="D124" s="0">
+        <v>6</v>
+      </c>
+      <c r="E124" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="G124" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>25</v>
+      </c>
+      <c r="B125" t="s">
+        <v>24</v>
+      </c>
+      <c r="C125">
+        <v>2026</v>
+      </c>
+      <c r="D125" s="0">
+        <v>6</v>
+      </c>
+      <c r="E125" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="G125" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>26</v>
+      </c>
+      <c r="B126" t="s">
+        <v>27</v>
+      </c>
+      <c r="C126">
+        <v>2026</v>
+      </c>
+      <c r="D126" s="0">
+        <v>6</v>
+      </c>
+      <c r="E126" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G126" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>28</v>
+      </c>
+      <c r="B127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C127">
+        <v>2026</v>
+      </c>
+      <c r="D127" s="0">
+        <v>6</v>
+      </c>
+      <c r="E127" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G127" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>29</v>
+      </c>
+      <c r="B128" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C128">
+        <v>2026</v>
+      </c>
+      <c r="D128" s="0">
+        <v>6</v>
+      </c>
+      <c r="E128" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G128" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>31</v>
+      </c>
+      <c r="B129" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C129">
+        <v>2026</v>
+      </c>
+      <c r="D129" s="0">
+        <v>6</v>
+      </c>
+      <c r="E129" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G129" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>32</v>
+      </c>
+      <c r="B130" t="s">
+        <v>33</v>
+      </c>
+      <c r="C130">
+        <v>2026</v>
+      </c>
+      <c r="D130" s="0">
+        <v>6</v>
+      </c>
+      <c r="E130" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G130" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>34</v>
+      </c>
+      <c r="B131" t="s">
+        <v>33</v>
+      </c>
+      <c r="C131">
+        <v>2026</v>
+      </c>
+      <c r="D131" s="0">
+        <v>6</v>
+      </c>
+      <c r="E131" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="G131" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>35</v>
+      </c>
+      <c r="B132" t="s">
+        <v>36</v>
+      </c>
+      <c r="C132">
+        <v>2026</v>
+      </c>
+      <c r="D132" s="0">
+        <v>6</v>
+      </c>
+      <c r="E132" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="G132" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>37</v>
+      </c>
+      <c r="B133" t="s">
+        <v>36</v>
+      </c>
+      <c r="C133">
+        <v>2026</v>
+      </c>
+      <c r="D133" s="0">
+        <v>6</v>
+      </c>
+      <c r="E133" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="G133" s="10" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated betting odds for last few races
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -428,6 +428,51 @@
   </si>
   <si>
     <t>9-2</t>
+  </si>
+  <si>
+    <t>23-20</t>
+  </si>
+  <si>
+    <t>14-5</t>
+  </si>
+  <si>
+    <t>8-1</t>
+  </si>
+  <si>
+    <t>161</t>
+  </si>
+  <si>
+    <t>110-1</t>
+  </si>
+  <si>
+    <t>7-2</t>
+  </si>
+  <si>
+    <t>7-1</t>
+  </si>
+  <si>
+    <t>16-4</t>
+  </si>
+  <si>
+    <t>125-1</t>
+  </si>
+  <si>
+    <t>5000-1</t>
+  </si>
+  <si>
+    <t>11-10</t>
+  </si>
+  <si>
+    <t>750-</t>
+  </si>
+  <si>
+    <t>7-4</t>
+  </si>
+  <si>
+    <t>21-10</t>
+  </si>
+  <si>
+    <t>40-1</t>
   </si>
 </sst>
 </file>
@@ -3618,6 +3663,1392 @@
         <v>122</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="s">
+        <v>5</v>
+      </c>
+      <c r="B134" t="s">
+        <v>6</v>
+      </c>
+      <c r="C134">
+        <v>2026</v>
+      </c>
+      <c r="D134" s="0">
+        <v>7</v>
+      </c>
+      <c r="E134" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F134" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s">
+        <v>7</v>
+      </c>
+      <c r="B135" t="s">
+        <v>6</v>
+      </c>
+      <c r="C135">
+        <v>2026</v>
+      </c>
+      <c r="D135" s="0">
+        <v>7</v>
+      </c>
+      <c r="E135" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F135" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s">
+        <v>8</v>
+      </c>
+      <c r="B136" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136">
+        <v>2026</v>
+      </c>
+      <c r="D136" s="0">
+        <v>7</v>
+      </c>
+      <c r="E136" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F136" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="s">
+        <v>10</v>
+      </c>
+      <c r="B137" t="s">
+        <v>9</v>
+      </c>
+      <c r="C137">
+        <v>2026</v>
+      </c>
+      <c r="D137" s="0">
+        <v>7</v>
+      </c>
+      <c r="E137" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="F137" s="10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="s">
+        <v>11</v>
+      </c>
+      <c r="B138" t="s">
+        <v>12</v>
+      </c>
+      <c r="C138">
+        <v>2026</v>
+      </c>
+      <c r="D138" s="0">
+        <v>7</v>
+      </c>
+      <c r="E138" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="F138" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="s">
+        <v>13</v>
+      </c>
+      <c r="B139" t="s">
+        <v>12</v>
+      </c>
+      <c r="C139">
+        <v>2026</v>
+      </c>
+      <c r="D139" s="0">
+        <v>7</v>
+      </c>
+      <c r="E139" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="F139" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s">
+        <v>14</v>
+      </c>
+      <c r="B140" t="s">
+        <v>15</v>
+      </c>
+      <c r="C140">
+        <v>2026</v>
+      </c>
+      <c r="D140" s="0">
+        <v>7</v>
+      </c>
+      <c r="E140" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F140" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
+        <v>16</v>
+      </c>
+      <c r="B141" t="s">
+        <v>15</v>
+      </c>
+      <c r="C141">
+        <v>2026</v>
+      </c>
+      <c r="D141" s="0">
+        <v>7</v>
+      </c>
+      <c r="E141" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F141" s="10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>17</v>
+      </c>
+      <c r="B142" t="s">
+        <v>18</v>
+      </c>
+      <c r="C142">
+        <v>2026</v>
+      </c>
+      <c r="D142" s="0">
+        <v>7</v>
+      </c>
+      <c r="E142" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F142" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s">
+        <v>19</v>
+      </c>
+      <c r="B143" t="s">
+        <v>18</v>
+      </c>
+      <c r="C143">
+        <v>2026</v>
+      </c>
+      <c r="D143" s="0">
+        <v>7</v>
+      </c>
+      <c r="E143" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F143" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="s">
+        <v>20</v>
+      </c>
+      <c r="B144" t="s">
+        <v>21</v>
+      </c>
+      <c r="C144">
+        <v>2026</v>
+      </c>
+      <c r="D144" s="0">
+        <v>7</v>
+      </c>
+      <c r="E144" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F144" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="s">
+        <v>22</v>
+      </c>
+      <c r="B145" t="s">
+        <v>21</v>
+      </c>
+      <c r="C145">
+        <v>2026</v>
+      </c>
+      <c r="D145" s="0">
+        <v>7</v>
+      </c>
+      <c r="E145" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F145" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="s">
+        <v>23</v>
+      </c>
+      <c r="B146" t="s">
+        <v>24</v>
+      </c>
+      <c r="C146">
+        <v>2026</v>
+      </c>
+      <c r="D146" s="0">
+        <v>7</v>
+      </c>
+      <c r="E146" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F146" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="s">
+        <v>25</v>
+      </c>
+      <c r="B147" t="s">
+        <v>24</v>
+      </c>
+      <c r="C147">
+        <v>2026</v>
+      </c>
+      <c r="D147" s="0">
+        <v>7</v>
+      </c>
+      <c r="E147" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F147" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="s">
+        <v>26</v>
+      </c>
+      <c r="B148" t="s">
+        <v>27</v>
+      </c>
+      <c r="C148">
+        <v>2026</v>
+      </c>
+      <c r="D148" s="0">
+        <v>7</v>
+      </c>
+      <c r="E148" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F148" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="s">
+        <v>28</v>
+      </c>
+      <c r="B149" t="s">
+        <v>27</v>
+      </c>
+      <c r="C149">
+        <v>2026</v>
+      </c>
+      <c r="D149" s="0">
+        <v>7</v>
+      </c>
+      <c r="E149" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F149" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="s">
+        <v>29</v>
+      </c>
+      <c r="B150" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C150">
+        <v>2026</v>
+      </c>
+      <c r="D150" s="0">
+        <v>7</v>
+      </c>
+      <c r="E150" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F150" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="s">
+        <v>31</v>
+      </c>
+      <c r="B151" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C151">
+        <v>2026</v>
+      </c>
+      <c r="D151" s="0">
+        <v>7</v>
+      </c>
+      <c r="E151" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F151" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="s">
+        <v>32</v>
+      </c>
+      <c r="B152" t="s">
+        <v>33</v>
+      </c>
+      <c r="C152">
+        <v>2026</v>
+      </c>
+      <c r="D152" s="0">
+        <v>7</v>
+      </c>
+      <c r="E152" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F152" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="s">
+        <v>34</v>
+      </c>
+      <c r="B153" t="s">
+        <v>33</v>
+      </c>
+      <c r="C153">
+        <v>2026</v>
+      </c>
+      <c r="D153" s="0">
+        <v>7</v>
+      </c>
+      <c r="E153" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F153" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="s">
+        <v>35</v>
+      </c>
+      <c r="B154" t="s">
+        <v>36</v>
+      </c>
+      <c r="C154">
+        <v>2026</v>
+      </c>
+      <c r="D154" s="0">
+        <v>7</v>
+      </c>
+      <c r="E154" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F154" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s">
+        <v>37</v>
+      </c>
+      <c r="B155" t="s">
+        <v>36</v>
+      </c>
+      <c r="C155">
+        <v>2026</v>
+      </c>
+      <c r="D155" s="0">
+        <v>7</v>
+      </c>
+      <c r="E155" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F155" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="s">
+        <v>5</v>
+      </c>
+      <c r="B156" t="s">
+        <v>6</v>
+      </c>
+      <c r="C156">
+        <v>2026</v>
+      </c>
+      <c r="D156" s="0">
+        <v>8</v>
+      </c>
+      <c r="E156" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="F156" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="H156" s="0" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="s">
+        <v>7</v>
+      </c>
+      <c r="B157" t="s">
+        <v>6</v>
+      </c>
+      <c r="C157">
+        <v>2026</v>
+      </c>
+      <c r="D157" s="0">
+        <v>8</v>
+      </c>
+      <c r="E157" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="H157" s="0" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="s">
+        <v>8</v>
+      </c>
+      <c r="B158" t="s">
+        <v>9</v>
+      </c>
+      <c r="C158">
+        <v>2026</v>
+      </c>
+      <c r="D158" s="0">
+        <v>8</v>
+      </c>
+      <c r="E158" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H158" s="0" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="s">
+        <v>10</v>
+      </c>
+      <c r="B159" t="s">
+        <v>9</v>
+      </c>
+      <c r="C159">
+        <v>2026</v>
+      </c>
+      <c r="D159" s="0">
+        <v>8</v>
+      </c>
+      <c r="E159" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="F159" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="H159" s="0" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s">
+        <v>11</v>
+      </c>
+      <c r="B160" t="s">
+        <v>12</v>
+      </c>
+      <c r="C160">
+        <v>2026</v>
+      </c>
+      <c r="D160" s="0">
+        <v>8</v>
+      </c>
+      <c r="E160" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="F160" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H160" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="s">
+        <v>13</v>
+      </c>
+      <c r="B161" t="s">
+        <v>12</v>
+      </c>
+      <c r="C161">
+        <v>2026</v>
+      </c>
+      <c r="D161" s="0">
+        <v>8</v>
+      </c>
+      <c r="E161" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="F161" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="H161" s="0" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="s">
+        <v>14</v>
+      </c>
+      <c r="B162" t="s">
+        <v>15</v>
+      </c>
+      <c r="C162">
+        <v>2026</v>
+      </c>
+      <c r="D162" s="0">
+        <v>8</v>
+      </c>
+      <c r="E162" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="F162" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="H162" s="0" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="s">
+        <v>16</v>
+      </c>
+      <c r="B163" t="s">
+        <v>15</v>
+      </c>
+      <c r="C163">
+        <v>2026</v>
+      </c>
+      <c r="D163" s="0">
+        <v>8</v>
+      </c>
+      <c r="E163" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="F163" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="H163" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>17</v>
+      </c>
+      <c r="B164" t="s">
+        <v>18</v>
+      </c>
+      <c r="C164">
+        <v>2026</v>
+      </c>
+      <c r="D164" s="0">
+        <v>8</v>
+      </c>
+      <c r="E164" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="F164" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="H164" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="s">
+        <v>19</v>
+      </c>
+      <c r="B165" t="s">
+        <v>18</v>
+      </c>
+      <c r="C165">
+        <v>2026</v>
+      </c>
+      <c r="D165" s="0">
+        <v>8</v>
+      </c>
+      <c r="E165" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="F165" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H165" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s">
+        <v>20</v>
+      </c>
+      <c r="B166" t="s">
+        <v>21</v>
+      </c>
+      <c r="C166">
+        <v>2026</v>
+      </c>
+      <c r="D166" s="0">
+        <v>8</v>
+      </c>
+      <c r="E166" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="F166" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H166" s="0" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s">
+        <v>22</v>
+      </c>
+      <c r="B167" t="s">
+        <v>21</v>
+      </c>
+      <c r="C167">
+        <v>2026</v>
+      </c>
+      <c r="D167" s="0">
+        <v>8</v>
+      </c>
+      <c r="E167" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F167" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H167" s="0" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="s">
+        <v>23</v>
+      </c>
+      <c r="B168" t="s">
+        <v>24</v>
+      </c>
+      <c r="C168">
+        <v>2026</v>
+      </c>
+      <c r="D168" s="0">
+        <v>8</v>
+      </c>
+      <c r="E168" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F168" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H168" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="s">
+        <v>25</v>
+      </c>
+      <c r="B169" t="s">
+        <v>24</v>
+      </c>
+      <c r="C169">
+        <v>2026</v>
+      </c>
+      <c r="D169" s="0">
+        <v>8</v>
+      </c>
+      <c r="E169" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F169" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H169" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="s">
+        <v>26</v>
+      </c>
+      <c r="B170" t="s">
+        <v>27</v>
+      </c>
+      <c r="C170">
+        <v>2026</v>
+      </c>
+      <c r="D170" s="0">
+        <v>8</v>
+      </c>
+      <c r="E170" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="F170" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H170" s="0" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="s">
+        <v>28</v>
+      </c>
+      <c r="B171" t="s">
+        <v>27</v>
+      </c>
+      <c r="C171">
+        <v>2026</v>
+      </c>
+      <c r="D171" s="0">
+        <v>8</v>
+      </c>
+      <c r="E171" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F171" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H171" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="s">
+        <v>29</v>
+      </c>
+      <c r="B172" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C172">
+        <v>2026</v>
+      </c>
+      <c r="D172" s="0">
+        <v>8</v>
+      </c>
+      <c r="E172" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F172" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H172" s="0" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s">
+        <v>31</v>
+      </c>
+      <c r="B173" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C173">
+        <v>2026</v>
+      </c>
+      <c r="D173" s="0">
+        <v>8</v>
+      </c>
+      <c r="E173" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F173" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H173" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="s">
+        <v>32</v>
+      </c>
+      <c r="B174" t="s">
+        <v>33</v>
+      </c>
+      <c r="C174">
+        <v>2026</v>
+      </c>
+      <c r="D174" s="0">
+        <v>8</v>
+      </c>
+      <c r="E174" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F174" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H174" s="0" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="s">
+        <v>34</v>
+      </c>
+      <c r="B175" t="s">
+        <v>33</v>
+      </c>
+      <c r="C175">
+        <v>2026</v>
+      </c>
+      <c r="D175" s="0">
+        <v>8</v>
+      </c>
+      <c r="E175" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F175" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H175" s="0" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s">
+        <v>35</v>
+      </c>
+      <c r="B176" t="s">
+        <v>36</v>
+      </c>
+      <c r="C176">
+        <v>2026</v>
+      </c>
+      <c r="D176" s="0">
+        <v>8</v>
+      </c>
+      <c r="E176" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="F176" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H176" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s">
+        <v>37</v>
+      </c>
+      <c r="B177" t="s">
+        <v>36</v>
+      </c>
+      <c r="C177">
+        <v>2026</v>
+      </c>
+      <c r="D177" s="0">
+        <v>8</v>
+      </c>
+      <c r="E177" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="F177" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H177" s="0" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s">
+        <v>5</v>
+      </c>
+      <c r="B178" t="s">
+        <v>6</v>
+      </c>
+      <c r="C178">
+        <v>2026</v>
+      </c>
+      <c r="D178" s="0">
+        <v>9</v>
+      </c>
+      <c r="E178" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F178" s="10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s">
+        <v>7</v>
+      </c>
+      <c r="B179" t="s">
+        <v>6</v>
+      </c>
+      <c r="C179">
+        <v>2026</v>
+      </c>
+      <c r="D179" s="0">
+        <v>9</v>
+      </c>
+      <c r="E179" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F179" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="s">
+        <v>8</v>
+      </c>
+      <c r="B180" t="s">
+        <v>9</v>
+      </c>
+      <c r="C180">
+        <v>2026</v>
+      </c>
+      <c r="D180" s="0">
+        <v>9</v>
+      </c>
+      <c r="E180" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F180" s="10" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="s">
+        <v>10</v>
+      </c>
+      <c r="B181" t="s">
+        <v>9</v>
+      </c>
+      <c r="C181">
+        <v>2026</v>
+      </c>
+      <c r="D181" s="0">
+        <v>9</v>
+      </c>
+      <c r="E181" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="F181" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s">
+        <v>11</v>
+      </c>
+      <c r="B182" t="s">
+        <v>12</v>
+      </c>
+      <c r="C182">
+        <v>2026</v>
+      </c>
+      <c r="D182" s="0">
+        <v>9</v>
+      </c>
+      <c r="E182" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F182" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="s">
+        <v>13</v>
+      </c>
+      <c r="B183" t="s">
+        <v>12</v>
+      </c>
+      <c r="C183">
+        <v>2026</v>
+      </c>
+      <c r="D183" s="0">
+        <v>9</v>
+      </c>
+      <c r="E183" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F183" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="s">
+        <v>14</v>
+      </c>
+      <c r="B184" t="s">
+        <v>15</v>
+      </c>
+      <c r="C184">
+        <v>2026</v>
+      </c>
+      <c r="D184" s="0">
+        <v>9</v>
+      </c>
+      <c r="E184" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="F184" s="10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="s">
+        <v>16</v>
+      </c>
+      <c r="B185" t="s">
+        <v>15</v>
+      </c>
+      <c r="C185">
+        <v>2026</v>
+      </c>
+      <c r="D185" s="0">
+        <v>9</v>
+      </c>
+      <c r="E185" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F185" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="s">
+        <v>17</v>
+      </c>
+      <c r="B186" t="s">
+        <v>18</v>
+      </c>
+      <c r="C186">
+        <v>2026</v>
+      </c>
+      <c r="D186" s="0">
+        <v>9</v>
+      </c>
+      <c r="E186" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F186" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="s">
+        <v>19</v>
+      </c>
+      <c r="B187" t="s">
+        <v>18</v>
+      </c>
+      <c r="C187">
+        <v>2026</v>
+      </c>
+      <c r="D187" s="0">
+        <v>9</v>
+      </c>
+      <c r="E187" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F187" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="s">
+        <v>20</v>
+      </c>
+      <c r="B188" t="s">
+        <v>21</v>
+      </c>
+      <c r="C188">
+        <v>2026</v>
+      </c>
+      <c r="D188" s="0">
+        <v>9</v>
+      </c>
+      <c r="E188" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F188" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="s">
+        <v>22</v>
+      </c>
+      <c r="B189" t="s">
+        <v>21</v>
+      </c>
+      <c r="C189">
+        <v>2026</v>
+      </c>
+      <c r="D189" s="0">
+        <v>9</v>
+      </c>
+      <c r="E189" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F189" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="s">
+        <v>23</v>
+      </c>
+      <c r="B190" t="s">
+        <v>24</v>
+      </c>
+      <c r="C190">
+        <v>2026</v>
+      </c>
+      <c r="D190" s="0">
+        <v>9</v>
+      </c>
+      <c r="E190" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F190" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="s">
+        <v>25</v>
+      </c>
+      <c r="B191" t="s">
+        <v>24</v>
+      </c>
+      <c r="C191">
+        <v>2026</v>
+      </c>
+      <c r="D191" s="0">
+        <v>9</v>
+      </c>
+      <c r="E191" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F191" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="s">
+        <v>26</v>
+      </c>
+      <c r="B192" t="s">
+        <v>27</v>
+      </c>
+      <c r="C192">
+        <v>2026</v>
+      </c>
+      <c r="D192" s="0">
+        <v>9</v>
+      </c>
+      <c r="E192" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F192" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="s">
+        <v>28</v>
+      </c>
+      <c r="B193" t="s">
+        <v>27</v>
+      </c>
+      <c r="C193">
+        <v>2026</v>
+      </c>
+      <c r="D193" s="0">
+        <v>9</v>
+      </c>
+      <c r="E193" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F193" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="s">
+        <v>29</v>
+      </c>
+      <c r="B194" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C194">
+        <v>2026</v>
+      </c>
+      <c r="D194" s="0">
+        <v>9</v>
+      </c>
+      <c r="E194" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F194" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="s">
+        <v>31</v>
+      </c>
+      <c r="B195" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C195">
+        <v>2026</v>
+      </c>
+      <c r="D195" s="0">
+        <v>9</v>
+      </c>
+      <c r="E195" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F195" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="s">
+        <v>32</v>
+      </c>
+      <c r="B196" t="s">
+        <v>33</v>
+      </c>
+      <c r="C196">
+        <v>2026</v>
+      </c>
+      <c r="D196" s="0">
+        <v>9</v>
+      </c>
+      <c r="E196" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F196" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="s">
+        <v>34</v>
+      </c>
+      <c r="B197" t="s">
+        <v>33</v>
+      </c>
+      <c r="C197">
+        <v>2026</v>
+      </c>
+      <c r="D197" s="0">
+        <v>9</v>
+      </c>
+      <c r="E197" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F197" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="s">
+        <v>35</v>
+      </c>
+      <c r="B198" t="s">
+        <v>36</v>
+      </c>
+      <c r="C198">
+        <v>2026</v>
+      </c>
+      <c r="D198" s="0">
+        <v>9</v>
+      </c>
+      <c r="E198" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F198" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="s">
+        <v>37</v>
+      </c>
+      <c r="B199" t="s">
+        <v>36</v>
+      </c>
+      <c r="C199">
+        <v>2026</v>
+      </c>
+      <c r="D199" s="0">
+        <v>9</v>
+      </c>
+      <c r="E199" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F199" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated data and selection after Silverstone
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -473,6 +473,15 @@
   </si>
   <si>
     <t>40-1</t>
+  </si>
+  <si>
+    <t>13-8</t>
+  </si>
+  <si>
+    <t>1304</t>
+  </si>
+  <si>
+    <t>13-4</t>
   </si>
 </sst>
 </file>
@@ -5049,6 +5058,446 @@
         <v>112</v>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="s">
+        <v>5</v>
+      </c>
+      <c r="B200" t="s">
+        <v>6</v>
+      </c>
+      <c r="C200">
+        <v>2026</v>
+      </c>
+      <c r="D200" s="0">
+        <v>10</v>
+      </c>
+      <c r="E200" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F200" s="10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="s">
+        <v>7</v>
+      </c>
+      <c r="B201" t="s">
+        <v>6</v>
+      </c>
+      <c r="C201">
+        <v>2026</v>
+      </c>
+      <c r="D201" s="0">
+        <v>10</v>
+      </c>
+      <c r="E201" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F201" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="s">
+        <v>8</v>
+      </c>
+      <c r="B202" t="s">
+        <v>9</v>
+      </c>
+      <c r="C202">
+        <v>2026</v>
+      </c>
+      <c r="D202" s="0">
+        <v>10</v>
+      </c>
+      <c r="E202" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="F202" s="10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="s">
+        <v>10</v>
+      </c>
+      <c r="B203" t="s">
+        <v>9</v>
+      </c>
+      <c r="C203">
+        <v>2026</v>
+      </c>
+      <c r="D203" s="0">
+        <v>10</v>
+      </c>
+      <c r="E203" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="F203" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="s">
+        <v>11</v>
+      </c>
+      <c r="B204" t="s">
+        <v>12</v>
+      </c>
+      <c r="C204">
+        <v>2026</v>
+      </c>
+      <c r="D204" s="0">
+        <v>10</v>
+      </c>
+      <c r="E204" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F204" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="s">
+        <v>13</v>
+      </c>
+      <c r="B205" t="s">
+        <v>12</v>
+      </c>
+      <c r="C205">
+        <v>2026</v>
+      </c>
+      <c r="D205" s="0">
+        <v>10</v>
+      </c>
+      <c r="E205" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="F205" s="10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="s">
+        <v>14</v>
+      </c>
+      <c r="B206" t="s">
+        <v>15</v>
+      </c>
+      <c r="C206">
+        <v>2026</v>
+      </c>
+      <c r="D206" s="0">
+        <v>10</v>
+      </c>
+      <c r="E206" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="F206" s="10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="s">
+        <v>16</v>
+      </c>
+      <c r="B207" t="s">
+        <v>15</v>
+      </c>
+      <c r="C207">
+        <v>2026</v>
+      </c>
+      <c r="D207" s="0">
+        <v>10</v>
+      </c>
+      <c r="E207" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F207" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="s">
+        <v>17</v>
+      </c>
+      <c r="B208" t="s">
+        <v>18</v>
+      </c>
+      <c r="C208">
+        <v>2026</v>
+      </c>
+      <c r="D208" s="0">
+        <v>10</v>
+      </c>
+      <c r="E208" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F208" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="s">
+        <v>19</v>
+      </c>
+      <c r="B209" t="s">
+        <v>18</v>
+      </c>
+      <c r="C209">
+        <v>2026</v>
+      </c>
+      <c r="D209" s="0">
+        <v>10</v>
+      </c>
+      <c r="E209" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F209" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="s">
+        <v>20</v>
+      </c>
+      <c r="B210" t="s">
+        <v>21</v>
+      </c>
+      <c r="C210">
+        <v>2026</v>
+      </c>
+      <c r="D210" s="0">
+        <v>10</v>
+      </c>
+      <c r="E210" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F210" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="s">
+        <v>22</v>
+      </c>
+      <c r="B211" t="s">
+        <v>21</v>
+      </c>
+      <c r="C211">
+        <v>2026</v>
+      </c>
+      <c r="D211" s="0">
+        <v>10</v>
+      </c>
+      <c r="E211" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F211" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="s">
+        <v>23</v>
+      </c>
+      <c r="B212" t="s">
+        <v>24</v>
+      </c>
+      <c r="C212">
+        <v>2026</v>
+      </c>
+      <c r="D212" s="0">
+        <v>10</v>
+      </c>
+      <c r="E212" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="F212" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="s">
+        <v>25</v>
+      </c>
+      <c r="B213" t="s">
+        <v>24</v>
+      </c>
+      <c r="C213">
+        <v>2026</v>
+      </c>
+      <c r="D213" s="0">
+        <v>10</v>
+      </c>
+      <c r="E213" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="F213" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="s">
+        <v>26</v>
+      </c>
+      <c r="B214" t="s">
+        <v>27</v>
+      </c>
+      <c r="C214">
+        <v>2026</v>
+      </c>
+      <c r="D214" s="0">
+        <v>10</v>
+      </c>
+      <c r="E214" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F214" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="s">
+        <v>28</v>
+      </c>
+      <c r="B215" t="s">
+        <v>27</v>
+      </c>
+      <c r="C215">
+        <v>2026</v>
+      </c>
+      <c r="D215" s="0">
+        <v>10</v>
+      </c>
+      <c r="E215" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F215" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="s">
+        <v>29</v>
+      </c>
+      <c r="B216" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C216">
+        <v>2026</v>
+      </c>
+      <c r="D216" s="0">
+        <v>10</v>
+      </c>
+      <c r="E216" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F216" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="s">
+        <v>31</v>
+      </c>
+      <c r="B217" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C217">
+        <v>2026</v>
+      </c>
+      <c r="D217" s="0">
+        <v>10</v>
+      </c>
+      <c r="E217" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F217" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="s">
+        <v>32</v>
+      </c>
+      <c r="B218" t="s">
+        <v>33</v>
+      </c>
+      <c r="C218">
+        <v>2026</v>
+      </c>
+      <c r="D218" s="0">
+        <v>10</v>
+      </c>
+      <c r="E218" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F218" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="s">
+        <v>34</v>
+      </c>
+      <c r="B219" t="s">
+        <v>33</v>
+      </c>
+      <c r="C219">
+        <v>2026</v>
+      </c>
+      <c r="D219" s="0">
+        <v>10</v>
+      </c>
+      <c r="E219" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F219" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="s">
+        <v>35</v>
+      </c>
+      <c r="B220" t="s">
+        <v>36</v>
+      </c>
+      <c r="C220">
+        <v>2026</v>
+      </c>
+      <c r="D220" s="0">
+        <v>10</v>
+      </c>
+      <c r="E220" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F220" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="s">
+        <v>37</v>
+      </c>
+      <c r="B221" t="s">
+        <v>36</v>
+      </c>
+      <c r="C221">
+        <v>2026</v>
+      </c>
+      <c r="D221" s="0">
+        <v>10</v>
+      </c>
+      <c r="E221" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F221" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated data and team selection for Hungary
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -482,6 +482,24 @@
   </si>
   <si>
     <t>13-4</t>
+  </si>
+  <si>
+    <t>4-6</t>
+  </si>
+  <si>
+    <t>23-4</t>
+  </si>
+  <si>
+    <t>22-1</t>
+  </si>
+  <si>
+    <t>600-1</t>
+  </si>
+  <si>
+    <t>4-1</t>
+  </si>
+  <si>
+    <t>3000</t>
   </si>
 </sst>
 </file>
@@ -5071,11 +5089,14 @@
       <c r="D200" s="0">
         <v>10</v>
       </c>
-      <c r="E200" s="10" t="s">
-        <v>126</v>
+      <c r="E200" s="0" t="s">
+        <v>118</v>
       </c>
       <c r="F200" s="10" t="s">
         <v>126</v>
+      </c>
+      <c r="H200" s="0" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="201">
@@ -5091,11 +5112,14 @@
       <c r="D201" s="0">
         <v>10</v>
       </c>
-      <c r="E201" s="10" t="s">
-        <v>153</v>
+      <c r="E201" s="0" t="s">
+        <v>159</v>
       </c>
       <c r="F201" s="10" t="s">
         <v>153</v>
+      </c>
+      <c r="H201" s="0" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="202">
@@ -5111,11 +5135,14 @@
       <c r="D202" s="0">
         <v>10</v>
       </c>
-      <c r="E202" s="10" t="s">
-        <v>156</v>
+      <c r="E202" s="0" t="s">
+        <v>136</v>
       </c>
       <c r="F202" s="10" t="s">
         <v>156</v>
+      </c>
+      <c r="H202" s="0" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="203">
@@ -5131,11 +5158,14 @@
       <c r="D203" s="0">
         <v>10</v>
       </c>
-      <c r="E203" s="10" t="s">
-        <v>154</v>
+      <c r="E203" s="0" t="s">
+        <v>157</v>
       </c>
       <c r="F203" s="10" t="s">
         <v>154</v>
+      </c>
+      <c r="H203" s="0" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="204">
@@ -5151,11 +5181,14 @@
       <c r="D204" s="0">
         <v>10</v>
       </c>
-      <c r="E204" s="10" t="s">
-        <v>135</v>
+      <c r="E204" s="0" t="s">
+        <v>158</v>
       </c>
       <c r="F204" s="10" t="s">
         <v>135</v>
+      </c>
+      <c r="H204" s="0" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="205">
@@ -5171,11 +5204,14 @@
       <c r="D205" s="0">
         <v>10</v>
       </c>
-      <c r="E205" s="10" t="s">
-        <v>110</v>
+      <c r="E205" s="0" t="s">
+        <v>102</v>
       </c>
       <c r="F205" s="10" t="s">
         <v>110</v>
+      </c>
+      <c r="H205" s="0" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="206">
@@ -5191,11 +5227,14 @@
       <c r="D206" s="0">
         <v>10</v>
       </c>
-      <c r="E206" s="10" t="s">
-        <v>144</v>
+      <c r="E206" s="0" t="s">
+        <v>93</v>
       </c>
       <c r="F206" s="10" t="s">
         <v>144</v>
+      </c>
+      <c r="H206" s="0" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="207">
@@ -5211,11 +5250,14 @@
       <c r="D207" s="0">
         <v>10</v>
       </c>
-      <c r="E207" s="10" t="s">
-        <v>97</v>
+      <c r="E207" s="0" t="s">
+        <v>115</v>
       </c>
       <c r="F207" s="10" t="s">
         <v>97</v>
+      </c>
+      <c r="H207" s="0" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="208">
@@ -5231,11 +5273,14 @@
       <c r="D208" s="0">
         <v>10</v>
       </c>
-      <c r="E208" s="10" t="s">
-        <v>120</v>
+      <c r="E208" s="0" t="s">
+        <v>112</v>
       </c>
       <c r="F208" s="10" t="s">
         <v>120</v>
+      </c>
+      <c r="H208" s="0" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="209">
@@ -5251,11 +5296,14 @@
       <c r="D209" s="0">
         <v>10</v>
       </c>
-      <c r="E209" s="10" t="s">
-        <v>112</v>
+      <c r="E209" s="0" t="s">
+        <v>120</v>
       </c>
       <c r="F209" s="10" t="s">
         <v>112</v>
+      </c>
+      <c r="H209" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="210">
@@ -5271,11 +5319,14 @@
       <c r="D210" s="0">
         <v>10</v>
       </c>
-      <c r="E210" s="10" t="s">
-        <v>101</v>
+      <c r="E210" s="0" t="s">
+        <v>160</v>
       </c>
       <c r="F210" s="10" t="s">
         <v>101</v>
+      </c>
+      <c r="H210" s="0" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="211">
@@ -5291,10 +5342,13 @@
       <c r="D211" s="0">
         <v>10</v>
       </c>
-      <c r="E211" s="10" t="s">
+      <c r="E211" s="0" t="s">
         <v>101</v>
       </c>
       <c r="F211" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="H211" s="0" t="s">
         <v>101</v>
       </c>
     </row>
@@ -5311,11 +5365,14 @@
       <c r="D212" s="0">
         <v>10</v>
       </c>
-      <c r="E212" s="10" t="s">
-        <v>148</v>
+      <c r="E212" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="F212" s="10" t="s">
         <v>148</v>
+      </c>
+      <c r="H212" s="0" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="213">
@@ -5331,10 +5388,13 @@
       <c r="D213" s="0">
         <v>10</v>
       </c>
-      <c r="E213" s="10" t="s">
+      <c r="E213" s="0" t="s">
         <v>148</v>
       </c>
       <c r="F213" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="H213" s="0" t="s">
         <v>148</v>
       </c>
     </row>
@@ -5351,10 +5411,13 @@
       <c r="D214" s="0">
         <v>10</v>
       </c>
-      <c r="E214" s="10" t="s">
+      <c r="E214" s="0" t="s">
         <v>120</v>
       </c>
       <c r="F214" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="H214" s="0" t="s">
         <v>120</v>
       </c>
     </row>
@@ -5371,11 +5434,14 @@
       <c r="D215" s="0">
         <v>10</v>
       </c>
-      <c r="E215" s="10" t="s">
-        <v>104</v>
+      <c r="E215" s="0" t="s">
+        <v>111</v>
       </c>
       <c r="F215" s="10" t="s">
         <v>104</v>
+      </c>
+      <c r="H215" s="0" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="216">
@@ -5391,10 +5457,13 @@
       <c r="D216" s="0">
         <v>10</v>
       </c>
-      <c r="E216" s="10" t="s">
+      <c r="E216" s="0" t="s">
         <v>100</v>
       </c>
       <c r="F216" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="H216" s="0" t="s">
         <v>100</v>
       </c>
     </row>
@@ -5411,10 +5480,13 @@
       <c r="D217" s="0">
         <v>10</v>
       </c>
-      <c r="E217" s="10" t="s">
+      <c r="E217" s="0" t="s">
         <v>100</v>
       </c>
       <c r="F217" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="H217" s="0" t="s">
         <v>100</v>
       </c>
     </row>
@@ -5431,11 +5503,14 @@
       <c r="D218" s="0">
         <v>10</v>
       </c>
-      <c r="E218" s="10" t="s">
-        <v>100</v>
+      <c r="E218" s="0" t="s">
+        <v>111</v>
       </c>
       <c r="F218" s="10" t="s">
         <v>100</v>
+      </c>
+      <c r="H218" s="0" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="219">
@@ -5451,11 +5526,14 @@
       <c r="D219" s="0">
         <v>10</v>
       </c>
-      <c r="E219" s="10" t="s">
-        <v>104</v>
+      <c r="E219" s="0" t="s">
+        <v>111</v>
       </c>
       <c r="F219" s="10" t="s">
         <v>104</v>
+      </c>
+      <c r="H219" s="0" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="220">
@@ -5471,10 +5549,13 @@
       <c r="D220" s="0">
         <v>10</v>
       </c>
-      <c r="E220" s="10" t="s">
+      <c r="E220" s="0" t="s">
         <v>103</v>
       </c>
       <c r="F220" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H220" s="0" t="s">
         <v>103</v>
       </c>
     </row>
@@ -5491,10 +5572,453 @@
       <c r="D221" s="0">
         <v>10</v>
       </c>
-      <c r="E221" s="10" t="s">
+      <c r="E221" s="0" t="s">
         <v>103</v>
       </c>
       <c r="F221" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H221" s="0" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="s">
+        <v>5</v>
+      </c>
+      <c r="B222" t="s">
+        <v>6</v>
+      </c>
+      <c r="C222">
+        <v>2026</v>
+      </c>
+      <c r="D222" s="0">
+        <v>11</v>
+      </c>
+      <c r="E222" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F222" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="s">
+        <v>7</v>
+      </c>
+      <c r="B223" t="s">
+        <v>6</v>
+      </c>
+      <c r="C223">
+        <v>2026</v>
+      </c>
+      <c r="D223" s="0">
+        <v>11</v>
+      </c>
+      <c r="E223" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F223" s="10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s">
+        <v>8</v>
+      </c>
+      <c r="B224" t="s">
+        <v>9</v>
+      </c>
+      <c r="C224">
+        <v>2026</v>
+      </c>
+      <c r="D224" s="0">
+        <v>11</v>
+      </c>
+      <c r="E224" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F224" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="s">
+        <v>10</v>
+      </c>
+      <c r="B225" t="s">
+        <v>9</v>
+      </c>
+      <c r="C225">
+        <v>2026</v>
+      </c>
+      <c r="D225" s="0">
+        <v>11</v>
+      </c>
+      <c r="E225" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="F225" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="s">
+        <v>11</v>
+      </c>
+      <c r="B226" t="s">
+        <v>12</v>
+      </c>
+      <c r="C226">
+        <v>2026</v>
+      </c>
+      <c r="D226" s="0">
+        <v>11</v>
+      </c>
+      <c r="E226" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F226" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="s">
+        <v>13</v>
+      </c>
+      <c r="B227" t="s">
+        <v>12</v>
+      </c>
+      <c r="C227">
+        <v>2026</v>
+      </c>
+      <c r="D227" s="0">
+        <v>11</v>
+      </c>
+      <c r="E227" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F227" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="s">
+        <v>14</v>
+      </c>
+      <c r="B228" t="s">
+        <v>15</v>
+      </c>
+      <c r="C228">
+        <v>2026</v>
+      </c>
+      <c r="D228" s="0">
+        <v>11</v>
+      </c>
+      <c r="E228" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F228" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="s">
+        <v>16</v>
+      </c>
+      <c r="B229" t="s">
+        <v>15</v>
+      </c>
+      <c r="C229">
+        <v>2026</v>
+      </c>
+      <c r="D229" s="0">
+        <v>11</v>
+      </c>
+      <c r="E229" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="F229" s="10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="s">
+        <v>17</v>
+      </c>
+      <c r="B230" t="s">
+        <v>18</v>
+      </c>
+      <c r="C230">
+        <v>2026</v>
+      </c>
+      <c r="D230" s="0">
+        <v>11</v>
+      </c>
+      <c r="E230" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F230" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="s">
+        <v>19</v>
+      </c>
+      <c r="B231" t="s">
+        <v>18</v>
+      </c>
+      <c r="C231">
+        <v>2026</v>
+      </c>
+      <c r="D231" s="0">
+        <v>11</v>
+      </c>
+      <c r="E231" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F231" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="s">
+        <v>20</v>
+      </c>
+      <c r="B232" t="s">
+        <v>21</v>
+      </c>
+      <c r="C232">
+        <v>2026</v>
+      </c>
+      <c r="D232" s="0">
+        <v>11</v>
+      </c>
+      <c r="E232" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F232" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="s">
+        <v>22</v>
+      </c>
+      <c r="B233" t="s">
+        <v>21</v>
+      </c>
+      <c r="C233">
+        <v>2026</v>
+      </c>
+      <c r="D233" s="0">
+        <v>11</v>
+      </c>
+      <c r="E233" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F233" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="s">
+        <v>23</v>
+      </c>
+      <c r="B234" t="s">
+        <v>24</v>
+      </c>
+      <c r="C234">
+        <v>2026</v>
+      </c>
+      <c r="D234" s="0">
+        <v>11</v>
+      </c>
+      <c r="E234" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F234" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="s">
+        <v>25</v>
+      </c>
+      <c r="B235" t="s">
+        <v>24</v>
+      </c>
+      <c r="C235">
+        <v>2026</v>
+      </c>
+      <c r="D235" s="0">
+        <v>11</v>
+      </c>
+      <c r="E235" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F235" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="s">
+        <v>26</v>
+      </c>
+      <c r="B236" t="s">
+        <v>27</v>
+      </c>
+      <c r="C236">
+        <v>2026</v>
+      </c>
+      <c r="D236" s="0">
+        <v>11</v>
+      </c>
+      <c r="E236" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F236" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="s">
+        <v>28</v>
+      </c>
+      <c r="B237" t="s">
+        <v>27</v>
+      </c>
+      <c r="C237">
+        <v>2026</v>
+      </c>
+      <c r="D237" s="0">
+        <v>11</v>
+      </c>
+      <c r="E237" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F237" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="s">
+        <v>29</v>
+      </c>
+      <c r="B238" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C238">
+        <v>2026</v>
+      </c>
+      <c r="D238" s="0">
+        <v>11</v>
+      </c>
+      <c r="E238" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F238" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="s">
+        <v>31</v>
+      </c>
+      <c r="B239" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C239">
+        <v>2026</v>
+      </c>
+      <c r="D239" s="0">
+        <v>11</v>
+      </c>
+      <c r="E239" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F239" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s">
+        <v>32</v>
+      </c>
+      <c r="B240" t="s">
+        <v>33</v>
+      </c>
+      <c r="C240">
+        <v>2026</v>
+      </c>
+      <c r="D240" s="0">
+        <v>11</v>
+      </c>
+      <c r="E240" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F240" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="s">
+        <v>34</v>
+      </c>
+      <c r="B241" t="s">
+        <v>33</v>
+      </c>
+      <c r="C241">
+        <v>2026</v>
+      </c>
+      <c r="D241" s="0">
+        <v>11</v>
+      </c>
+      <c r="E241" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F241" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="s">
+        <v>35</v>
+      </c>
+      <c r="B242" t="s">
+        <v>36</v>
+      </c>
+      <c r="C242">
+        <v>2026</v>
+      </c>
+      <c r="D242" s="0">
+        <v>11</v>
+      </c>
+      <c r="E242" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F242" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="s">
+        <v>37</v>
+      </c>
+      <c r="B243" t="s">
+        <v>36</v>
+      </c>
+      <c r="C243">
+        <v>2026</v>
+      </c>
+      <c r="D243" s="0">
+        <v>11</v>
+      </c>
+      <c r="E243" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F243" s="10" t="s">
         <v>103</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated betting odds after FP2
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -500,6 +500,9 @@
   </si>
   <si>
     <t>3000</t>
+  </si>
+  <si>
+    <t>5-2</t>
   </si>
 </sst>
 </file>
@@ -5595,11 +5598,14 @@
       <c r="D222" s="0">
         <v>11</v>
       </c>
-      <c r="E222" s="10" t="s">
-        <v>93</v>
+      <c r="E222" s="0" t="s">
+        <v>138</v>
       </c>
       <c r="F222" s="10" t="s">
         <v>93</v>
+      </c>
+      <c r="H222" s="0" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="223">
@@ -5615,11 +5621,14 @@
       <c r="D223" s="0">
         <v>11</v>
       </c>
-      <c r="E223" s="10" t="s">
-        <v>126</v>
+      <c r="E223" s="0" t="s">
+        <v>159</v>
       </c>
       <c r="F223" s="10" t="s">
         <v>126</v>
+      </c>
+      <c r="H223" s="0" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="224">
@@ -5635,11 +5644,14 @@
       <c r="D224" s="0">
         <v>11</v>
       </c>
-      <c r="E224" s="10" t="s">
-        <v>136</v>
+      <c r="E224" s="0" t="s">
+        <v>116</v>
       </c>
       <c r="F224" s="10" t="s">
         <v>136</v>
+      </c>
+      <c r="H224" s="0" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="225">
@@ -5655,11 +5667,14 @@
       <c r="D225" s="0">
         <v>11</v>
       </c>
-      <c r="E225" s="10" t="s">
-        <v>151</v>
+      <c r="E225" s="0" t="s">
+        <v>123</v>
       </c>
       <c r="F225" s="10" t="s">
         <v>151</v>
+      </c>
+      <c r="H225" s="0" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="226">
@@ -5675,11 +5690,14 @@
       <c r="D226" s="0">
         <v>11</v>
       </c>
-      <c r="E226" s="10" t="s">
-        <v>94</v>
+      <c r="E226" s="0" t="s">
+        <v>115</v>
       </c>
       <c r="F226" s="10" t="s">
         <v>94</v>
+      </c>
+      <c r="H226" s="0" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="227">
@@ -5695,11 +5713,14 @@
       <c r="D227" s="0">
         <v>11</v>
       </c>
-      <c r="E227" s="10" t="s">
-        <v>147</v>
+      <c r="E227" s="0" t="s">
+        <v>110</v>
       </c>
       <c r="F227" s="10" t="s">
         <v>147</v>
+      </c>
+      <c r="H227" s="0" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="228">
@@ -5715,11 +5736,14 @@
       <c r="D228" s="0">
         <v>11</v>
       </c>
-      <c r="E228" s="10" t="s">
-        <v>161</v>
+      <c r="E228" s="0" t="s">
+        <v>163</v>
       </c>
       <c r="F228" s="10" t="s">
         <v>161</v>
+      </c>
+      <c r="H228" s="0" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="229">
@@ -5735,11 +5759,14 @@
       <c r="D229" s="0">
         <v>11</v>
       </c>
-      <c r="E229" s="10" t="s">
-        <v>138</v>
+      <c r="E229" s="0" t="s">
+        <v>161</v>
       </c>
       <c r="F229" s="10" t="s">
         <v>138</v>
+      </c>
+      <c r="H229" s="0" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="230">
@@ -5755,11 +5782,14 @@
       <c r="D230" s="0">
         <v>11</v>
       </c>
-      <c r="E230" s="10" t="s">
-        <v>112</v>
+      <c r="E230" s="0" t="s">
+        <v>120</v>
       </c>
       <c r="F230" s="10" t="s">
         <v>112</v>
+      </c>
+      <c r="H230" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="231">
@@ -5775,11 +5805,14 @@
       <c r="D231" s="0">
         <v>11</v>
       </c>
-      <c r="E231" s="10" t="s">
-        <v>111</v>
+      <c r="E231" s="0" t="s">
+        <v>120</v>
       </c>
       <c r="F231" s="10" t="s">
         <v>111</v>
+      </c>
+      <c r="H231" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="232">
@@ -5795,10 +5828,13 @@
       <c r="D232" s="0">
         <v>11</v>
       </c>
-      <c r="E232" s="10" t="s">
+      <c r="E232" s="0" t="s">
         <v>100</v>
       </c>
       <c r="F232" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="H232" s="0" t="s">
         <v>100</v>
       </c>
     </row>
@@ -5816,10 +5852,13 @@
         <v>11</v>
       </c>
       <c r="E233" s="10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F233" s="10" t="s">
         <v>100</v>
+      </c>
+      <c r="H233" s="10" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="234">
@@ -5835,11 +5874,14 @@
       <c r="D234" s="0">
         <v>11</v>
       </c>
-      <c r="E234" s="10" t="s">
-        <v>111</v>
+      <c r="E234" s="0" t="s">
+        <v>112</v>
       </c>
       <c r="F234" s="10" t="s">
         <v>111</v>
+      </c>
+      <c r="H234" s="0" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="235">
@@ -5855,11 +5897,14 @@
       <c r="D235" s="0">
         <v>11</v>
       </c>
-      <c r="E235" s="10" t="s">
-        <v>112</v>
+      <c r="E235" s="0" t="s">
+        <v>103</v>
       </c>
       <c r="F235" s="10" t="s">
         <v>112</v>
+      </c>
+      <c r="H235" s="0" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="236">
@@ -5875,10 +5920,13 @@
       <c r="D236" s="0">
         <v>11</v>
       </c>
-      <c r="E236" s="10" t="s">
+      <c r="E236" s="0" t="s">
         <v>112</v>
       </c>
       <c r="F236" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="H236" s="0" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5895,11 +5943,14 @@
       <c r="D237" s="0">
         <v>11</v>
       </c>
-      <c r="E237" s="10" t="s">
-        <v>111</v>
+      <c r="E237" s="0" t="s">
+        <v>112</v>
       </c>
       <c r="F237" s="10" t="s">
         <v>111</v>
+      </c>
+      <c r="H237" s="0" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="238">
@@ -5921,6 +5972,9 @@
       <c r="F238" s="10" t="s">
         <v>104</v>
       </c>
+      <c r="H238" s="10" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="s">
@@ -5941,6 +5995,9 @@
       <c r="F239" s="10" t="s">
         <v>104</v>
       </c>
+      <c r="H239" s="10" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="s">
@@ -5955,11 +6012,14 @@
       <c r="D240" s="0">
         <v>11</v>
       </c>
-      <c r="E240" s="10" t="s">
-        <v>104</v>
+      <c r="E240" s="0" t="s">
+        <v>112</v>
       </c>
       <c r="F240" s="10" t="s">
         <v>104</v>
+      </c>
+      <c r="H240" s="0" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="241">
@@ -5975,11 +6035,14 @@
       <c r="D241" s="0">
         <v>11</v>
       </c>
-      <c r="E241" s="10" t="s">
-        <v>104</v>
+      <c r="E241" s="0" t="s">
+        <v>112</v>
       </c>
       <c r="F241" s="10" t="s">
         <v>104</v>
+      </c>
+      <c r="H241" s="0" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="242">
@@ -5995,11 +6058,14 @@
       <c r="D242" s="0">
         <v>11</v>
       </c>
-      <c r="E242" s="10" t="s">
-        <v>103</v>
+      <c r="E242" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="F242" s="10" t="s">
         <v>103</v>
+      </c>
+      <c r="H242" s="0" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="243">
@@ -6015,11 +6081,14 @@
       <c r="D243" s="0">
         <v>11</v>
       </c>
-      <c r="E243" s="10" t="s">
-        <v>103</v>
+      <c r="E243" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="F243" s="10" t="s">
         <v>103</v>
+      </c>
+      <c r="H243" s="0" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Betting odds for R13
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3211,6 +3211,15 @@
   </si>
   <si>
     <t>TSU</t>
+  </si>
+  <si>
+    <t>57-17</t>
+  </si>
+  <si>
+    <t>800-1</t>
+  </si>
+  <si>
+    <t>979-1</t>
   </si>
 </sst>
 </file>
@@ -9386,6 +9395,446 @@
         <v>106</v>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="s">
+        <v>955</v>
+      </c>
+      <c r="B266" t="s">
+        <v>956</v>
+      </c>
+      <c r="C266">
+        <v>2026</v>
+      </c>
+      <c r="D266" s="0">
+        <v>13</v>
+      </c>
+      <c r="E266" s="0" t="s">
+        <v>497</v>
+      </c>
+      <c r="H266" s="0" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="s">
+        <v>960</v>
+      </c>
+      <c r="B267" t="s">
+        <v>961</v>
+      </c>
+      <c r="C267">
+        <v>2026</v>
+      </c>
+      <c r="D267" s="0">
+        <v>13</v>
+      </c>
+      <c r="E267" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="H267" s="0" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="s">
+        <v>965</v>
+      </c>
+      <c r="B268" t="s">
+        <v>966</v>
+      </c>
+      <c r="C268">
+        <v>2026</v>
+      </c>
+      <c r="D268" s="0">
+        <v>13</v>
+      </c>
+      <c r="E268" s="0" t="s">
+        <v>771</v>
+      </c>
+      <c r="H268" s="0" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="s">
+        <v>970</v>
+      </c>
+      <c r="B269" t="s">
+        <v>971</v>
+      </c>
+      <c r="C269">
+        <v>2026</v>
+      </c>
+      <c r="D269" s="0">
+        <v>13</v>
+      </c>
+      <c r="E269" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="H269" s="0" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="s">
+        <v>975</v>
+      </c>
+      <c r="B270" t="s">
+        <v>976</v>
+      </c>
+      <c r="C270">
+        <v>2026</v>
+      </c>
+      <c r="D270" s="0">
+        <v>13</v>
+      </c>
+      <c r="E270" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="H270" s="0" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="18" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B271" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C271">
+        <v>2026</v>
+      </c>
+      <c r="D271" s="0">
+        <v>13</v>
+      </c>
+      <c r="E271" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H271" s="0" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="s">
+        <v>985</v>
+      </c>
+      <c r="B272" t="s">
+        <v>986</v>
+      </c>
+      <c r="C272">
+        <v>2026</v>
+      </c>
+      <c r="D272" s="0">
+        <v>13</v>
+      </c>
+      <c r="E272" s="0" t="s">
+        <v>497</v>
+      </c>
+      <c r="H272" s="0" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="s">
+        <v>990</v>
+      </c>
+      <c r="B273" t="s">
+        <v>991</v>
+      </c>
+      <c r="C273">
+        <v>2026</v>
+      </c>
+      <c r="D273" s="0">
+        <v>13</v>
+      </c>
+      <c r="E273" s="0" t="s">
+        <v>1066</v>
+      </c>
+      <c r="H273" s="0" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="s">
+        <v>995</v>
+      </c>
+      <c r="B274" t="s">
+        <v>996</v>
+      </c>
+      <c r="C274">
+        <v>2026</v>
+      </c>
+      <c r="D274" s="0">
+        <v>13</v>
+      </c>
+      <c r="E274" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="H274" s="0" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B275" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C275">
+        <v>2026</v>
+      </c>
+      <c r="D275" s="0">
+        <v>13</v>
+      </c>
+      <c r="E275" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="H275" s="0" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="18" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B276" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C276">
+        <v>2026</v>
+      </c>
+      <c r="D276" s="0">
+        <v>13</v>
+      </c>
+      <c r="E276" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H276" s="0" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B277" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C277">
+        <v>2026</v>
+      </c>
+      <c r="D277" s="0">
+        <v>13</v>
+      </c>
+      <c r="E277" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H277" s="0" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B278" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C278">
+        <v>2026</v>
+      </c>
+      <c r="D278" s="0">
+        <v>13</v>
+      </c>
+      <c r="E278" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="H278" s="0" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B279" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C279">
+        <v>2026</v>
+      </c>
+      <c r="D279" s="0">
+        <v>13</v>
+      </c>
+      <c r="E279" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="H279" s="0" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B280" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C280">
+        <v>2026</v>
+      </c>
+      <c r="D280" s="0">
+        <v>13</v>
+      </c>
+      <c r="E280" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="H280" s="0" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B281" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C281">
+        <v>2026</v>
+      </c>
+      <c r="D281" s="0">
+        <v>13</v>
+      </c>
+      <c r="E281" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="H281" s="0" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B282" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C282">
+        <v>2026</v>
+      </c>
+      <c r="D282" s="0">
+        <v>13</v>
+      </c>
+      <c r="E282" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="H282" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B283" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C283">
+        <v>2026</v>
+      </c>
+      <c r="D283" s="0">
+        <v>13</v>
+      </c>
+      <c r="E283" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="H283" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B284" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C284">
+        <v>2026</v>
+      </c>
+      <c r="D284" s="0">
+        <v>13</v>
+      </c>
+      <c r="E284" s="0" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H284" s="0" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B285" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C285">
+        <v>2026</v>
+      </c>
+      <c r="D285" s="0">
+        <v>13</v>
+      </c>
+      <c r="E285" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="H285" s="0" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B286" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C286">
+        <v>2026</v>
+      </c>
+      <c r="D286" s="0">
+        <v>13</v>
+      </c>
+      <c r="E286" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="H286" s="0" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B287" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C287">
+        <v>2026</v>
+      </c>
+      <c r="D287" s="0">
+        <v>13</v>
+      </c>
+      <c r="E287" s="0" t="s">
+        <v>345</v>
+      </c>
+      <c r="H287" s="0" t="s">
+        <v>345</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated stats after race 13
</commit_message>
<xml_diff>
--- a/data/f1_betting_odds.xlsx
+++ b/data/f1_betting_odds.xlsx
@@ -3220,6 +3220,9 @@
   </si>
   <si>
     <t>979-1</t>
+  </si>
+  <si>
+    <t>19-5</t>
   </si>
 </sst>
 </file>
@@ -9835,6 +9838,446 @@
         <v>345</v>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="s">
+        <v>955</v>
+      </c>
+      <c r="B288" t="s">
+        <v>956</v>
+      </c>
+      <c r="C288">
+        <v>2026</v>
+      </c>
+      <c r="D288" s="0">
+        <v>14</v>
+      </c>
+      <c r="E288" s="10" t="s">
+        <v>1069</v>
+      </c>
+      <c r="F288" s="10" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="s">
+        <v>960</v>
+      </c>
+      <c r="B289" t="s">
+        <v>961</v>
+      </c>
+      <c r="C289">
+        <v>2026</v>
+      </c>
+      <c r="D289" s="0">
+        <v>14</v>
+      </c>
+      <c r="E289" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="F289" s="10" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="s">
+        <v>965</v>
+      </c>
+      <c r="B290" t="s">
+        <v>966</v>
+      </c>
+      <c r="C290">
+        <v>2026</v>
+      </c>
+      <c r="D290" s="0">
+        <v>14</v>
+      </c>
+      <c r="E290" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F290" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="s">
+        <v>970</v>
+      </c>
+      <c r="B291" t="s">
+        <v>971</v>
+      </c>
+      <c r="C291">
+        <v>2026</v>
+      </c>
+      <c r="D291" s="0">
+        <v>14</v>
+      </c>
+      <c r="E291" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="F291" s="10" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="s">
+        <v>975</v>
+      </c>
+      <c r="B292" t="s">
+        <v>976</v>
+      </c>
+      <c r="C292">
+        <v>2026</v>
+      </c>
+      <c r="D292" s="0">
+        <v>14</v>
+      </c>
+      <c r="E292" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="F292" s="10" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="18" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B293" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C293">
+        <v>2026</v>
+      </c>
+      <c r="D293" s="0">
+        <v>14</v>
+      </c>
+      <c r="E293" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F293" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="s">
+        <v>985</v>
+      </c>
+      <c r="B294" t="s">
+        <v>986</v>
+      </c>
+      <c r="C294">
+        <v>2026</v>
+      </c>
+      <c r="D294" s="0">
+        <v>14</v>
+      </c>
+      <c r="E294" s="10" t="s">
+        <v>577</v>
+      </c>
+      <c r="F294" s="10" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="s">
+        <v>990</v>
+      </c>
+      <c r="B295" t="s">
+        <v>991</v>
+      </c>
+      <c r="C295">
+        <v>2026</v>
+      </c>
+      <c r="D295" s="0">
+        <v>14</v>
+      </c>
+      <c r="E295" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F295" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="s">
+        <v>995</v>
+      </c>
+      <c r="B296" t="s">
+        <v>996</v>
+      </c>
+      <c r="C296">
+        <v>2026</v>
+      </c>
+      <c r="D296" s="0">
+        <v>14</v>
+      </c>
+      <c r="E296" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F296" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B297" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C297">
+        <v>2026</v>
+      </c>
+      <c r="D297" s="0">
+        <v>14</v>
+      </c>
+      <c r="E297" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F297" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="18" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B298" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C298">
+        <v>2026</v>
+      </c>
+      <c r="D298" s="0">
+        <v>14</v>
+      </c>
+      <c r="E298" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="F298" s="10" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B299" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C299">
+        <v>2026</v>
+      </c>
+      <c r="D299" s="0">
+        <v>14</v>
+      </c>
+      <c r="E299" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F299" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B300" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C300">
+        <v>2026</v>
+      </c>
+      <c r="D300" s="0">
+        <v>14</v>
+      </c>
+      <c r="E300" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F300" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B301" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C301">
+        <v>2026</v>
+      </c>
+      <c r="D301" s="0">
+        <v>14</v>
+      </c>
+      <c r="E301" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F301" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B302" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C302">
+        <v>2026</v>
+      </c>
+      <c r="D302" s="0">
+        <v>14</v>
+      </c>
+      <c r="E302" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F302" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B303" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C303">
+        <v>2026</v>
+      </c>
+      <c r="D303" s="0">
+        <v>14</v>
+      </c>
+      <c r="E303" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F303" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B304" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C304">
+        <v>2026</v>
+      </c>
+      <c r="D304" s="0">
+        <v>14</v>
+      </c>
+      <c r="E304" s="10" t="s">
+        <v>897</v>
+      </c>
+      <c r="F304" s="10" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B305" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C305">
+        <v>2026</v>
+      </c>
+      <c r="D305" s="0">
+        <v>14</v>
+      </c>
+      <c r="E305" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F305" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B306" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C306">
+        <v>2026</v>
+      </c>
+      <c r="D306" s="0">
+        <v>14</v>
+      </c>
+      <c r="E306" s="10" t="s">
+        <v>1067</v>
+      </c>
+      <c r="F306" s="10" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B307" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C307">
+        <v>2026</v>
+      </c>
+      <c r="D307" s="0">
+        <v>14</v>
+      </c>
+      <c r="E307" s="10" t="s">
+        <v>897</v>
+      </c>
+      <c r="F307" s="10" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B308" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C308">
+        <v>2026</v>
+      </c>
+      <c r="D308" s="0">
+        <v>14</v>
+      </c>
+      <c r="E308" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F308" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B309" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C309">
+        <v>2026</v>
+      </c>
+      <c r="D309" s="0">
+        <v>14</v>
+      </c>
+      <c r="E309" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F309" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>